<commit_message>
krds color 값 변경 중
</commit_message>
<xml_diff>
--- a/doc/금융감독원 홈페이지_UIUX_퍼블_컴포넌트리스트 .xlsx
+++ b/doc/금융감독원 홈페이지_UIUX_퍼블_컴포넌트리스트 .xlsx
@@ -8,16 +8,19 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\03.Publishing\fss\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F93260AC-0D20-45ED-99CC-47945DC6DC78}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3388EF8B-1D84-44CF-8529-6044779B968A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="-5100" windowWidth="29040" windowHeight="15720" tabRatio="499" activeTab="1" xr2:uid="{BA3ED54C-CC85-4CD0-8ADB-46ECF631616A}"/>
+    <workbookView xWindow="46260" yWindow="-4680" windowWidth="20115" windowHeight="15105" tabRatio="499" activeTab="3" xr2:uid="{BA3ED54C-CC85-4CD0-8ADB-46ECF631616A}"/>
   </bookViews>
   <sheets>
     <sheet name="체크리스트_목록" sheetId="1" r:id="rId1"/>
     <sheet name="ia guide" sheetId="2" r:id="rId2"/>
+    <sheet name="design guide" sheetId="4" r:id="rId3"/>
+    <sheet name="Sheet3" sheetId="5" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'ia guide'!$A$4:$G$119</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'design guide'!$A$4:$G$115</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'ia guide'!$A$4:$G$116</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">체크리스트_목록!$A$4:$F$164</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
@@ -30,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="375" uniqueCount="204">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="526" uniqueCount="214">
   <si>
     <t>대분류</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -830,6 +833,46 @@
 font.css
 common.css
 content.css</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>02.20.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Identifier</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Masthead</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Disabled</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Pressed</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Hover</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Default</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>.krds-btn.link.basic</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>.krds-btn.link</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>color: var(--krds-button--color-link-text)</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -3183,7 +3226,7 @@
   <sheetPr>
     <tabColor theme="5" tint="0.59999389629810485"/>
   </sheetPr>
-  <dimension ref="A1:I165"/>
+  <dimension ref="A1:I162"/>
   <sheetFormatPr defaultRowHeight="17" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="21.25" customWidth="1"/>
@@ -3258,103 +3301,119 @@
       <c r="C6" s="13" t="s">
         <v>130</v>
       </c>
-      <c r="D6" s="15"/>
+      <c r="D6" s="15" t="s">
+        <v>206</v>
+      </c>
       <c r="E6" s="23"/>
-      <c r="F6" s="23"/>
+      <c r="F6" s="16" t="s">
+        <v>204</v>
+      </c>
       <c r="G6" s="19"/>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A7" s="39"/>
       <c r="B7" s="36"/>
-      <c r="C7" s="35" t="s">
+      <c r="C7" s="13" t="s">
         <v>7</v>
       </c>
       <c r="D7" s="15" t="s">
-        <v>90</v>
+        <v>205</v>
       </c>
       <c r="E7" s="23"/>
-      <c r="F7" s="23"/>
+      <c r="F7" s="16" t="s">
+        <v>204</v>
+      </c>
       <c r="G7" s="19"/>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:8" ht="34" x14ac:dyDescent="0.45">
       <c r="A8" s="39"/>
       <c r="B8" s="36"/>
-      <c r="C8" s="37"/>
+      <c r="C8" s="35" t="s">
+        <v>191</v>
+      </c>
       <c r="D8" s="15" t="s">
-        <v>95</v>
-      </c>
-      <c r="E8" s="23"/>
-      <c r="F8" s="23"/>
-      <c r="G8" s="19"/>
-    </row>
-    <row r="9" spans="1:8" ht="34" x14ac:dyDescent="0.45">
+        <v>88</v>
+      </c>
+      <c r="E8" s="24"/>
+      <c r="F8" s="16" t="s">
+        <v>204</v>
+      </c>
+      <c r="G8" s="17" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A9" s="39"/>
       <c r="B9" s="36"/>
-      <c r="C9" s="35" t="s">
-        <v>191</v>
-      </c>
-      <c r="D9" s="15" t="s">
-        <v>88</v>
-      </c>
-      <c r="E9" s="24"/>
-      <c r="F9" s="24"/>
-      <c r="G9" s="17" t="s">
-        <v>139</v>
-      </c>
+      <c r="C9" s="36"/>
+      <c r="D9" s="15"/>
+      <c r="E9" s="15"/>
+      <c r="F9" s="15"/>
+      <c r="G9" s="19"/>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A10" s="39"/>
       <c r="B10" s="36"/>
-      <c r="C10" s="36"/>
-      <c r="D10" s="15"/>
-      <c r="E10" s="15"/>
-      <c r="F10" s="15"/>
+      <c r="C10" s="35" t="s">
+        <v>192</v>
+      </c>
+      <c r="D10" s="17" t="s">
+        <v>87</v>
+      </c>
+      <c r="E10" s="24"/>
+      <c r="F10" s="24"/>
       <c r="G10" s="19"/>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A11" s="39"/>
       <c r="B11" s="36"/>
-      <c r="C11" s="35" t="s">
-        <v>192</v>
-      </c>
-      <c r="D11" s="17" t="s">
-        <v>87</v>
-      </c>
-      <c r="E11" s="24"/>
-      <c r="F11" s="24"/>
+      <c r="C11" s="36"/>
+      <c r="D11" s="17"/>
+      <c r="E11" s="17"/>
+      <c r="F11" s="17"/>
       <c r="G11" s="19"/>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A12" s="39"/>
-      <c r="B12" s="36"/>
-      <c r="C12" s="36"/>
-      <c r="D12" s="17"/>
-      <c r="E12" s="17"/>
-      <c r="F12" s="17"/>
+      <c r="B12" s="35" t="s">
+        <v>6</v>
+      </c>
+      <c r="C12" s="13" t="s">
+        <v>10</v>
+      </c>
+      <c r="D12" s="18" t="s">
+        <v>107</v>
+      </c>
+      <c r="E12" s="25"/>
+      <c r="F12" s="16" t="s">
+        <v>204</v>
+      </c>
       <c r="G12" s="19"/>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A13" s="39"/>
-      <c r="B13" s="35" t="s">
-        <v>6</v>
-      </c>
+      <c r="B13" s="36"/>
       <c r="C13" s="35" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D13" s="18" t="s">
-        <v>107</v>
+        <v>59</v>
       </c>
       <c r="E13" s="25"/>
-      <c r="F13" s="25"/>
+      <c r="F13" s="16" t="s">
+        <v>204</v>
+      </c>
       <c r="G13" s="19"/>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A14" s="39"/>
       <c r="B14" s="36"/>
       <c r="C14" s="36"/>
-      <c r="D14" s="18"/>
-      <c r="E14" s="18"/>
-      <c r="F14" s="18"/>
+      <c r="D14" s="18" t="s">
+        <v>60</v>
+      </c>
+      <c r="E14" s="25"/>
+      <c r="F14" s="25"/>
       <c r="G14" s="19"/>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.45">
@@ -3369,141 +3428,145 @@
     <row r="16" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A16" s="39"/>
       <c r="B16" s="36"/>
-      <c r="C16" s="35" t="s">
-        <v>11</v>
+      <c r="C16" s="13" t="s">
+        <v>12</v>
       </c>
       <c r="D16" s="18" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="E16" s="25"/>
-      <c r="F16" s="25"/>
+      <c r="F16" s="16" t="s">
+        <v>204</v>
+      </c>
       <c r="G16" s="19"/>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A17" s="39"/>
       <c r="B17" s="36"/>
-      <c r="C17" s="36"/>
-      <c r="D17" s="18" t="s">
-        <v>60</v>
-      </c>
-      <c r="E17" s="25"/>
-      <c r="F17" s="25"/>
+      <c r="C17" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="D17" s="15" t="s">
+        <v>58</v>
+      </c>
+      <c r="E17" s="23"/>
+      <c r="F17" s="16" t="s">
+        <v>204</v>
+      </c>
       <c r="G17" s="19"/>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A18" s="39"/>
       <c r="B18" s="36"/>
-      <c r="C18" s="37"/>
-      <c r="D18" s="18"/>
-      <c r="E18" s="18"/>
-      <c r="F18" s="18"/>
+      <c r="C18" s="35" t="s">
+        <v>14</v>
+      </c>
+      <c r="D18" s="15"/>
+      <c r="E18" s="15"/>
+      <c r="F18" s="15"/>
       <c r="G18" s="19"/>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A19" s="39"/>
       <c r="B19" s="36"/>
-      <c r="C19" s="13" t="s">
-        <v>12</v>
-      </c>
-      <c r="D19" s="18" t="s">
-        <v>63</v>
-      </c>
-      <c r="E19" s="25"/>
-      <c r="F19" s="25"/>
+      <c r="C19" s="36"/>
+      <c r="D19" s="15"/>
+      <c r="E19" s="15"/>
+      <c r="F19" s="15"/>
       <c r="G19" s="19"/>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A20" s="39"/>
       <c r="B20" s="36"/>
-      <c r="C20" s="13" t="s">
-        <v>13</v>
-      </c>
-      <c r="D20" s="15" t="s">
-        <v>58</v>
-      </c>
-      <c r="E20" s="23" t="s">
-        <v>131</v>
-      </c>
-      <c r="F20" s="23"/>
+      <c r="C20" s="36"/>
+      <c r="D20" s="15"/>
+      <c r="E20" s="15"/>
+      <c r="F20" s="15"/>
       <c r="G20" s="19"/>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A21" s="39"/>
       <c r="B21" s="36"/>
-      <c r="C21" s="35" t="s">
-        <v>14</v>
-      </c>
-      <c r="D21" s="15"/>
-      <c r="E21" s="15"/>
-      <c r="F21" s="15"/>
+      <c r="C21" s="37"/>
+      <c r="D21" s="19"/>
+      <c r="E21" s="19"/>
+      <c r="F21" s="19"/>
       <c r="G21" s="19"/>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A22" s="39"/>
       <c r="B22" s="36"/>
-      <c r="C22" s="36"/>
-      <c r="D22" s="15"/>
-      <c r="E22" s="15"/>
-      <c r="F22" s="15"/>
+      <c r="C22" s="35" t="s">
+        <v>15</v>
+      </c>
+      <c r="D22" s="19" t="s">
+        <v>91</v>
+      </c>
+      <c r="E22" s="16" t="s">
+        <v>133</v>
+      </c>
+      <c r="F22" s="16"/>
       <c r="G22" s="19"/>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A23" s="39"/>
       <c r="B23" s="36"/>
       <c r="C23" s="36"/>
-      <c r="D23" s="15"/>
-      <c r="E23" s="15"/>
-      <c r="F23" s="15"/>
+      <c r="D23" s="20" t="s">
+        <v>98</v>
+      </c>
+      <c r="E23" s="14"/>
+      <c r="F23" s="14"/>
       <c r="G23" s="19"/>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A24" s="39"/>
       <c r="B24" s="36"/>
-      <c r="C24" s="37"/>
-      <c r="D24" s="19"/>
-      <c r="E24" s="19"/>
-      <c r="F24" s="19"/>
+      <c r="C24" s="36"/>
+      <c r="D24" s="21"/>
+      <c r="E24" s="21"/>
+      <c r="F24" s="21"/>
       <c r="G24" s="19"/>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A25" s="39"/>
-      <c r="B25" s="36"/>
-      <c r="C25" s="35" t="s">
-        <v>15</v>
-      </c>
-      <c r="D25" s="19" t="s">
-        <v>91</v>
-      </c>
-      <c r="E25" s="16" t="s">
-        <v>133</v>
-      </c>
-      <c r="F25" s="16"/>
+      <c r="B25" s="37"/>
+      <c r="C25" s="37"/>
+      <c r="D25" s="21"/>
+      <c r="E25" s="21"/>
+      <c r="F25" s="21"/>
       <c r="G25" s="19"/>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A26" s="39"/>
-      <c r="B26" s="36"/>
-      <c r="C26" s="36"/>
-      <c r="D26" s="20" t="s">
-        <v>98</v>
-      </c>
-      <c r="E26" s="14"/>
-      <c r="F26" s="14"/>
+      <c r="B26" s="35" t="s">
+        <v>16</v>
+      </c>
+      <c r="C26" s="35" t="s">
+        <v>24</v>
+      </c>
+      <c r="D26" s="21" t="s">
+        <v>110</v>
+      </c>
+      <c r="E26" s="26"/>
+      <c r="F26" s="26"/>
       <c r="G26" s="19"/>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A27" s="39"/>
       <c r="B27" s="36"/>
       <c r="C27" s="36"/>
-      <c r="D27" s="21"/>
-      <c r="E27" s="21"/>
-      <c r="F27" s="21"/>
+      <c r="D27" s="21" t="s">
+        <v>111</v>
+      </c>
+      <c r="E27" s="26"/>
+      <c r="F27" s="26"/>
       <c r="G27" s="19"/>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A28" s="39"/>
-      <c r="B28" s="37"/>
-      <c r="C28" s="37"/>
+      <c r="B28" s="36"/>
+      <c r="C28" s="36"/>
       <c r="D28" s="21"/>
       <c r="E28" s="21"/>
       <c r="F28" s="21"/>
@@ -3511,14 +3574,12 @@
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A29" s="39"/>
-      <c r="B29" s="35" t="s">
-        <v>16</v>
-      </c>
+      <c r="B29" s="36"/>
       <c r="C29" s="35" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D29" s="21" t="s">
-        <v>110</v>
+        <v>79</v>
       </c>
       <c r="E29" s="26"/>
       <c r="F29" s="26"/>
@@ -3528,17 +3589,15 @@
       <c r="A30" s="39"/>
       <c r="B30" s="36"/>
       <c r="C30" s="36"/>
-      <c r="D30" s="21" t="s">
-        <v>111</v>
-      </c>
-      <c r="E30" s="26"/>
-      <c r="F30" s="26"/>
+      <c r="D30" s="21"/>
+      <c r="E30" s="21"/>
+      <c r="F30" s="21"/>
       <c r="G30" s="19"/>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A31" s="39"/>
       <c r="B31" s="36"/>
-      <c r="C31" s="36"/>
+      <c r="C31" s="37"/>
       <c r="D31" s="21"/>
       <c r="E31" s="21"/>
       <c r="F31" s="21"/>
@@ -3548,13 +3607,11 @@
       <c r="A32" s="39"/>
       <c r="B32" s="36"/>
       <c r="C32" s="35" t="s">
-        <v>25</v>
-      </c>
-      <c r="D32" s="21" t="s">
-        <v>79</v>
-      </c>
-      <c r="E32" s="26"/>
-      <c r="F32" s="26"/>
+        <v>26</v>
+      </c>
+      <c r="D32" s="21"/>
+      <c r="E32" s="21"/>
+      <c r="F32" s="21"/>
       <c r="G32" s="19"/>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.45">
@@ -3569,7 +3626,7 @@
     <row r="34" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A34" s="39"/>
       <c r="B34" s="36"/>
-      <c r="C34" s="37"/>
+      <c r="C34" s="36"/>
       <c r="D34" s="21"/>
       <c r="E34" s="21"/>
       <c r="F34" s="21"/>
@@ -3578,9 +3635,7 @@
     <row r="35" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A35" s="39"/>
       <c r="B35" s="36"/>
-      <c r="C35" s="35" t="s">
-        <v>26</v>
-      </c>
+      <c r="C35" s="37"/>
       <c r="D35" s="21"/>
       <c r="E35" s="21"/>
       <c r="F35" s="21"/>
@@ -3589,16 +3644,20 @@
     <row r="36" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A36" s="39"/>
       <c r="B36" s="36"/>
-      <c r="C36" s="36"/>
-      <c r="D36" s="21"/>
-      <c r="E36" s="21"/>
-      <c r="F36" s="21"/>
+      <c r="C36" s="35" t="s">
+        <v>27</v>
+      </c>
+      <c r="D36" s="21" t="s">
+        <v>84</v>
+      </c>
+      <c r="E36" s="26"/>
+      <c r="F36" s="26"/>
       <c r="G36" s="19"/>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A37" s="39"/>
       <c r="B37" s="36"/>
-      <c r="C37" s="36"/>
+      <c r="C37" s="37"/>
       <c r="D37" s="21"/>
       <c r="E37" s="21"/>
       <c r="F37" s="21"/>
@@ -3607,20 +3666,22 @@
     <row r="38" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A38" s="39"/>
       <c r="B38" s="36"/>
-      <c r="C38" s="37"/>
-      <c r="D38" s="21"/>
-      <c r="E38" s="21"/>
-      <c r="F38" s="21"/>
+      <c r="C38" s="35" t="s">
+        <v>28</v>
+      </c>
+      <c r="D38" s="21" t="s">
+        <v>96</v>
+      </c>
+      <c r="E38" s="26"/>
+      <c r="F38" s="26"/>
       <c r="G38" s="19"/>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A39" s="39"/>
       <c r="B39" s="36"/>
-      <c r="C39" s="35" t="s">
-        <v>27</v>
-      </c>
+      <c r="C39" s="36"/>
       <c r="D39" s="21" t="s">
-        <v>84</v>
+        <v>97</v>
       </c>
       <c r="E39" s="26"/>
       <c r="F39" s="26"/>
@@ -3629,20 +3690,22 @@
     <row r="40" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A40" s="39"/>
       <c r="B40" s="36"/>
-      <c r="C40" s="37"/>
-      <c r="D40" s="21"/>
-      <c r="E40" s="21"/>
-      <c r="F40" s="21"/>
+      <c r="C40" s="35" t="s">
+        <v>29</v>
+      </c>
+      <c r="D40" s="21" t="s">
+        <v>80</v>
+      </c>
+      <c r="E40" s="26"/>
+      <c r="F40" s="26"/>
       <c r="G40" s="19"/>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A41" s="39"/>
       <c r="B41" s="36"/>
-      <c r="C41" s="35" t="s">
-        <v>28</v>
-      </c>
+      <c r="C41" s="36"/>
       <c r="D41" s="21" t="s">
-        <v>96</v>
+        <v>81</v>
       </c>
       <c r="E41" s="26"/>
       <c r="F41" s="26"/>
@@ -3651,9 +3714,9 @@
     <row r="42" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A42" s="39"/>
       <c r="B42" s="36"/>
-      <c r="C42" s="36"/>
+      <c r="C42" s="37"/>
       <c r="D42" s="21" t="s">
-        <v>97</v>
+        <v>82</v>
       </c>
       <c r="E42" s="26"/>
       <c r="F42" s="26"/>
@@ -3663,10 +3726,10 @@
       <c r="A43" s="39"/>
       <c r="B43" s="36"/>
       <c r="C43" s="35" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D43" s="21" t="s">
-        <v>80</v>
+        <v>61</v>
       </c>
       <c r="E43" s="26"/>
       <c r="F43" s="26"/>
@@ -3677,7 +3740,7 @@
       <c r="B44" s="36"/>
       <c r="C44" s="36"/>
       <c r="D44" s="21" t="s">
-        <v>81</v>
+        <v>62</v>
       </c>
       <c r="E44" s="26"/>
       <c r="F44" s="26"/>
@@ -3687,55 +3750,53 @@
       <c r="A45" s="39"/>
       <c r="B45" s="36"/>
       <c r="C45" s="37"/>
-      <c r="D45" s="21" t="s">
-        <v>82</v>
-      </c>
-      <c r="E45" s="26"/>
-      <c r="F45" s="26"/>
+      <c r="D45" s="21"/>
+      <c r="E45" s="21"/>
+      <c r="F45" s="21"/>
       <c r="G45" s="19"/>
     </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A46" s="39"/>
       <c r="B46" s="36"/>
       <c r="C46" s="35" t="s">
-        <v>30</v>
-      </c>
-      <c r="D46" s="21" t="s">
-        <v>61</v>
-      </c>
-      <c r="E46" s="26"/>
-      <c r="F46" s="26"/>
+        <v>31</v>
+      </c>
+      <c r="D46" s="21"/>
+      <c r="E46" s="21"/>
+      <c r="F46" s="21"/>
       <c r="G46" s="19"/>
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A47" s="39"/>
       <c r="B47" s="36"/>
       <c r="C47" s="36"/>
-      <c r="D47" s="21" t="s">
-        <v>62</v>
-      </c>
-      <c r="E47" s="26"/>
-      <c r="F47" s="26"/>
+      <c r="D47" s="21"/>
+      <c r="E47" s="21"/>
+      <c r="F47" s="21"/>
       <c r="G47" s="19"/>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A48" s="39"/>
       <c r="B48" s="36"/>
-      <c r="C48" s="37"/>
-      <c r="D48" s="21"/>
-      <c r="E48" s="21"/>
-      <c r="F48" s="21"/>
+      <c r="C48" s="35" t="s">
+        <v>32</v>
+      </c>
+      <c r="D48" s="21" t="s">
+        <v>72</v>
+      </c>
+      <c r="E48" s="26"/>
+      <c r="F48" s="26"/>
       <c r="G48" s="19"/>
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A49" s="39"/>
       <c r="B49" s="36"/>
-      <c r="C49" s="35" t="s">
-        <v>31</v>
-      </c>
-      <c r="D49" s="21"/>
-      <c r="E49" s="21"/>
-      <c r="F49" s="21"/>
+      <c r="C49" s="36"/>
+      <c r="D49" s="21" t="s">
+        <v>73</v>
+      </c>
+      <c r="E49" s="26"/>
+      <c r="F49" s="26"/>
       <c r="G49" s="19"/>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.45">
@@ -3751,10 +3812,10 @@
       <c r="A51" s="39"/>
       <c r="B51" s="36"/>
       <c r="C51" s="35" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="D51" s="21" t="s">
-        <v>72</v>
+        <v>112</v>
       </c>
       <c r="E51" s="26"/>
       <c r="F51" s="26"/>
@@ -3764,11 +3825,9 @@
       <c r="A52" s="39"/>
       <c r="B52" s="36"/>
       <c r="C52" s="36"/>
-      <c r="D52" s="21" t="s">
-        <v>73</v>
-      </c>
-      <c r="E52" s="26"/>
-      <c r="F52" s="26"/>
+      <c r="D52" s="21"/>
+      <c r="E52" s="21"/>
+      <c r="F52" s="21"/>
       <c r="G52" s="19"/>
     </row>
     <row r="53" spans="1:7" x14ac:dyDescent="0.45">
@@ -3784,10 +3843,10 @@
       <c r="A54" s="39"/>
       <c r="B54" s="36"/>
       <c r="C54" s="35" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D54" s="21" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="E54" s="26"/>
       <c r="F54" s="26"/>
@@ -3796,7 +3855,7 @@
     <row r="55" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A55" s="39"/>
       <c r="B55" s="36"/>
-      <c r="C55" s="36"/>
+      <c r="C55" s="37"/>
       <c r="D55" s="21"/>
       <c r="E55" s="21"/>
       <c r="F55" s="21"/>
@@ -3805,20 +3864,22 @@
     <row r="56" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A56" s="39"/>
       <c r="B56" s="36"/>
-      <c r="C56" s="36"/>
-      <c r="D56" s="21"/>
-      <c r="E56" s="21"/>
-      <c r="F56" s="21"/>
+      <c r="C56" s="35" t="s">
+        <v>35</v>
+      </c>
+      <c r="D56" s="21" t="s">
+        <v>120</v>
+      </c>
+      <c r="E56" s="26"/>
+      <c r="F56" s="26"/>
       <c r="G56" s="19"/>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A57" s="39"/>
-      <c r="B57" s="36"/>
-      <c r="C57" s="35" t="s">
-        <v>34</v>
-      </c>
+      <c r="B57" s="37"/>
+      <c r="C57" s="36"/>
       <c r="D57" s="21" t="s">
-        <v>113</v>
+        <v>121</v>
       </c>
       <c r="E57" s="26"/>
       <c r="F57" s="26"/>
@@ -3826,47 +3887,51 @@
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A58" s="39"/>
-      <c r="B58" s="36"/>
-      <c r="C58" s="37"/>
-      <c r="D58" s="21"/>
-      <c r="E58" s="21"/>
-      <c r="F58" s="21"/>
+      <c r="B58" s="35" t="s">
+        <v>17</v>
+      </c>
+      <c r="C58" s="35" t="s">
+        <v>36</v>
+      </c>
+      <c r="D58" s="15" t="s">
+        <v>94</v>
+      </c>
+      <c r="E58" s="23"/>
+      <c r="F58" s="16" t="s">
+        <v>135</v>
+      </c>
       <c r="G58" s="19"/>
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A59" s="39"/>
       <c r="B59" s="36"/>
-      <c r="C59" s="35" t="s">
-        <v>35</v>
-      </c>
-      <c r="D59" s="21" t="s">
-        <v>120</v>
-      </c>
-      <c r="E59" s="26"/>
-      <c r="F59" s="26"/>
+      <c r="C59" s="36"/>
+      <c r="D59" s="15"/>
+      <c r="E59" s="15"/>
+      <c r="F59" s="16"/>
       <c r="G59" s="19"/>
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A60" s="39"/>
-      <c r="B60" s="37"/>
-      <c r="C60" s="36"/>
-      <c r="D60" s="21" t="s">
-        <v>121</v>
-      </c>
-      <c r="E60" s="26"/>
-      <c r="F60" s="26"/>
+      <c r="B60" s="36"/>
+      <c r="C60" s="35" t="s">
+        <v>37</v>
+      </c>
+      <c r="D60" s="15" t="s">
+        <v>64</v>
+      </c>
+      <c r="E60" s="23"/>
+      <c r="F60" s="16" t="s">
+        <v>135</v>
+      </c>
       <c r="G60" s="19"/>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A61" s="39"/>
-      <c r="B61" s="35" t="s">
-        <v>17</v>
-      </c>
-      <c r="C61" s="35" t="s">
-        <v>36</v>
-      </c>
+      <c r="B61" s="36"/>
+      <c r="C61" s="36"/>
       <c r="D61" s="15" t="s">
-        <v>94</v>
+        <v>65</v>
       </c>
       <c r="E61" s="23"/>
       <c r="F61" s="16" t="s">
@@ -3878,19 +3943,21 @@
       <c r="A62" s="39"/>
       <c r="B62" s="36"/>
       <c r="C62" s="36"/>
-      <c r="D62" s="15"/>
-      <c r="E62" s="15"/>
-      <c r="F62" s="16"/>
+      <c r="D62" s="15" t="s">
+        <v>66</v>
+      </c>
+      <c r="E62" s="23"/>
+      <c r="F62" s="16" t="s">
+        <v>135</v>
+      </c>
       <c r="G62" s="19"/>
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A63" s="39"/>
       <c r="B63" s="36"/>
-      <c r="C63" s="35" t="s">
-        <v>37</v>
-      </c>
+      <c r="C63" s="36"/>
       <c r="D63" s="15" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="E63" s="23"/>
       <c r="F63" s="16" t="s">
@@ -3903,7 +3970,7 @@
       <c r="B64" s="36"/>
       <c r="C64" s="36"/>
       <c r="D64" s="15" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="E64" s="23"/>
       <c r="F64" s="16" t="s">
@@ -3916,7 +3983,7 @@
       <c r="B65" s="36"/>
       <c r="C65" s="36"/>
       <c r="D65" s="15" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="E65" s="23"/>
       <c r="F65" s="16" t="s">
@@ -3926,10 +3993,14 @@
     </row>
     <row r="66" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A66" s="39"/>
-      <c r="B66" s="36"/>
-      <c r="C66" s="36"/>
+      <c r="B66" s="35" t="s">
+        <v>18</v>
+      </c>
+      <c r="C66" s="35" t="s">
+        <v>38</v>
+      </c>
       <c r="D66" s="15" t="s">
-        <v>67</v>
+        <v>99</v>
       </c>
       <c r="E66" s="23"/>
       <c r="F66" s="16" t="s">
@@ -3942,7 +4013,7 @@
       <c r="B67" s="36"/>
       <c r="C67" s="36"/>
       <c r="D67" s="15" t="s">
-        <v>68</v>
+        <v>100</v>
       </c>
       <c r="E67" s="23"/>
       <c r="F67" s="16" t="s">
@@ -3955,7 +4026,7 @@
       <c r="B68" s="36"/>
       <c r="C68" s="36"/>
       <c r="D68" s="15" t="s">
-        <v>69</v>
+        <v>101</v>
       </c>
       <c r="E68" s="23"/>
       <c r="F68" s="16" t="s">
@@ -3965,14 +4036,12 @@
     </row>
     <row r="69" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A69" s="39"/>
-      <c r="B69" s="35" t="s">
-        <v>18</v>
-      </c>
+      <c r="B69" s="36"/>
       <c r="C69" s="35" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="D69" s="15" t="s">
-        <v>99</v>
+        <v>74</v>
       </c>
       <c r="E69" s="23"/>
       <c r="F69" s="16" t="s">
@@ -3985,7 +4054,7 @@
       <c r="B70" s="36"/>
       <c r="C70" s="36"/>
       <c r="D70" s="15" t="s">
-        <v>100</v>
+        <v>75</v>
       </c>
       <c r="E70" s="23"/>
       <c r="F70" s="16" t="s">
@@ -3998,7 +4067,7 @@
       <c r="B71" s="36"/>
       <c r="C71" s="36"/>
       <c r="D71" s="15" t="s">
-        <v>101</v>
+        <v>76</v>
       </c>
       <c r="E71" s="23"/>
       <c r="F71" s="16" t="s">
@@ -4006,55 +4075,53 @@
       </c>
       <c r="G71" s="19"/>
     </row>
-    <row r="72" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="72" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A72" s="39"/>
       <c r="B72" s="36"/>
       <c r="C72" s="35" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D72" s="15" t="s">
-        <v>74</v>
+        <v>103</v>
       </c>
       <c r="E72" s="23"/>
       <c r="F72" s="16" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="G72" s="19"/>
     </row>
-    <row r="73" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="73" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A73" s="39"/>
       <c r="B73" s="36"/>
       <c r="C73" s="36"/>
       <c r="D73" s="15" t="s">
-        <v>75</v>
+        <v>104</v>
       </c>
       <c r="E73" s="23"/>
       <c r="F73" s="16" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="G73" s="19"/>
     </row>
-    <row r="74" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="74" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A74" s="39"/>
       <c r="B74" s="36"/>
       <c r="C74" s="36"/>
       <c r="D74" s="15" t="s">
-        <v>76</v>
+        <v>105</v>
       </c>
       <c r="E74" s="23"/>
       <c r="F74" s="16" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="G74" s="19"/>
     </row>
     <row r="75" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A75" s="39"/>
       <c r="B75" s="36"/>
-      <c r="C75" s="35" t="s">
-        <v>40</v>
-      </c>
+      <c r="C75" s="36"/>
       <c r="D75" s="15" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="E75" s="23"/>
       <c r="F75" s="16" t="s">
@@ -4065,9 +4132,11 @@
     <row r="76" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A76" s="39"/>
       <c r="B76" s="36"/>
-      <c r="C76" s="36"/>
+      <c r="C76" s="35" t="s">
+        <v>41</v>
+      </c>
       <c r="D76" s="15" t="s">
-        <v>104</v>
+        <v>114</v>
       </c>
       <c r="E76" s="23"/>
       <c r="F76" s="16" t="s">
@@ -4080,7 +4149,7 @@
       <c r="B77" s="36"/>
       <c r="C77" s="36"/>
       <c r="D77" s="15" t="s">
-        <v>105</v>
+        <v>115</v>
       </c>
       <c r="E77" s="23"/>
       <c r="F77" s="16" t="s">
@@ -4091,9 +4160,11 @@
     <row r="78" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A78" s="39"/>
       <c r="B78" s="36"/>
-      <c r="C78" s="36"/>
+      <c r="C78" s="35" t="s">
+        <v>42</v>
+      </c>
       <c r="D78" s="15" t="s">
-        <v>106</v>
+        <v>134</v>
       </c>
       <c r="E78" s="23"/>
       <c r="F78" s="16" t="s">
@@ -4104,11 +4175,9 @@
     <row r="79" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A79" s="39"/>
       <c r="B79" s="36"/>
-      <c r="C79" s="35" t="s">
-        <v>41</v>
-      </c>
+      <c r="C79" s="36"/>
       <c r="D79" s="15" t="s">
-        <v>114</v>
+        <v>124</v>
       </c>
       <c r="E79" s="23"/>
       <c r="F79" s="16" t="s">
@@ -4116,87 +4185,79 @@
       </c>
       <c r="G79" s="19"/>
     </row>
-    <row r="80" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="80" spans="1:7" ht="15.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A80" s="39"/>
-      <c r="B80" s="36"/>
-      <c r="C80" s="36"/>
-      <c r="D80" s="15" t="s">
-        <v>115</v>
-      </c>
-      <c r="E80" s="23"/>
-      <c r="F80" s="16" t="s">
-        <v>136</v>
-      </c>
+      <c r="B80" s="35" t="s">
+        <v>19</v>
+      </c>
+      <c r="C80" s="35" t="s">
+        <v>43</v>
+      </c>
+      <c r="D80" s="21" t="s">
+        <v>109</v>
+      </c>
+      <c r="E80" s="26"/>
+      <c r="F80" s="26"/>
       <c r="G80" s="19"/>
     </row>
     <row r="81" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A81" s="39"/>
       <c r="B81" s="36"/>
-      <c r="C81" s="35" t="s">
-        <v>42</v>
-      </c>
-      <c r="D81" s="15" t="s">
-        <v>134</v>
-      </c>
-      <c r="E81" s="23"/>
-      <c r="F81" s="16" t="s">
-        <v>136</v>
-      </c>
+      <c r="C81" s="37"/>
+      <c r="D81" s="15"/>
+      <c r="E81" s="15"/>
+      <c r="F81" s="15"/>
       <c r="G81" s="19"/>
     </row>
     <row r="82" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A82" s="39"/>
       <c r="B82" s="36"/>
-      <c r="C82" s="36"/>
+      <c r="C82" s="35" t="s">
+        <v>44</v>
+      </c>
       <c r="D82" s="15" t="s">
-        <v>124</v>
+        <v>108</v>
       </c>
       <c r="E82" s="23"/>
-      <c r="F82" s="16" t="s">
-        <v>136</v>
-      </c>
+      <c r="F82" s="23"/>
       <c r="G82" s="19"/>
     </row>
-    <row r="83" spans="1:7" ht="15.5" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="83" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A83" s="39"/>
-      <c r="B83" s="35" t="s">
-        <v>19</v>
-      </c>
-      <c r="C83" s="35" t="s">
-        <v>43</v>
-      </c>
-      <c r="D83" s="21" t="s">
-        <v>109</v>
-      </c>
-      <c r="E83" s="26"/>
-      <c r="F83" s="26"/>
+      <c r="B83" s="37"/>
+      <c r="C83" s="37"/>
+      <c r="D83" s="15"/>
+      <c r="E83" s="15"/>
+      <c r="F83" s="15"/>
       <c r="G83" s="19"/>
     </row>
     <row r="84" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A84" s="39"/>
-      <c r="B84" s="36"/>
-      <c r="C84" s="37"/>
-      <c r="D84" s="15"/>
-      <c r="E84" s="15"/>
-      <c r="F84" s="15"/>
+      <c r="B84" s="35" t="s">
+        <v>20</v>
+      </c>
+      <c r="C84" s="35" t="s">
+        <v>45</v>
+      </c>
+      <c r="D84" s="15" t="s">
+        <v>89</v>
+      </c>
+      <c r="E84" s="23"/>
+      <c r="F84" s="23"/>
       <c r="G84" s="19"/>
     </row>
     <row r="85" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A85" s="39"/>
       <c r="B85" s="36"/>
-      <c r="C85" s="35" t="s">
-        <v>44</v>
-      </c>
-      <c r="D85" s="15" t="s">
-        <v>108</v>
-      </c>
-      <c r="E85" s="23"/>
-      <c r="F85" s="23"/>
+      <c r="C85" s="36"/>
+      <c r="D85" s="15"/>
+      <c r="E85" s="15"/>
+      <c r="F85" s="15"/>
       <c r="G85" s="19"/>
     </row>
     <row r="86" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A86" s="39"/>
-      <c r="B86" s="37"/>
+      <c r="B86" s="36"/>
       <c r="C86" s="37"/>
       <c r="D86" s="15"/>
       <c r="E86" s="15"/>
@@ -4205,14 +4266,12 @@
     </row>
     <row r="87" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A87" s="39"/>
-      <c r="B87" s="35" t="s">
-        <v>20</v>
-      </c>
+      <c r="B87" s="36"/>
       <c r="C87" s="35" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="D87" s="15" t="s">
-        <v>89</v>
+        <v>128</v>
       </c>
       <c r="E87" s="23"/>
       <c r="F87" s="23"/>
@@ -4230,64 +4289,66 @@
     <row r="89" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A89" s="39"/>
       <c r="B89" s="36"/>
-      <c r="C89" s="37"/>
-      <c r="D89" s="15"/>
-      <c r="E89" s="15"/>
-      <c r="F89" s="15"/>
+      <c r="C89" s="35" t="s">
+        <v>47</v>
+      </c>
+      <c r="D89" s="15" t="s">
+        <v>78</v>
+      </c>
+      <c r="E89" s="23"/>
+      <c r="F89" s="23"/>
       <c r="G89" s="19"/>
     </row>
     <row r="90" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A90" s="39"/>
       <c r="B90" s="36"/>
-      <c r="C90" s="35" t="s">
-        <v>46</v>
-      </c>
-      <c r="D90" s="15" t="s">
-        <v>128</v>
-      </c>
-      <c r="E90" s="23"/>
-      <c r="F90" s="23"/>
+      <c r="C90" s="36"/>
+      <c r="D90" s="15"/>
+      <c r="E90" s="15"/>
+      <c r="F90" s="15"/>
       <c r="G90" s="19"/>
     </row>
     <row r="91" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A91" s="39"/>
       <c r="B91" s="36"/>
-      <c r="C91" s="36"/>
-      <c r="D91" s="15"/>
-      <c r="E91" s="15"/>
-      <c r="F91" s="15"/>
+      <c r="C91" s="35" t="s">
+        <v>48</v>
+      </c>
+      <c r="D91" s="15" t="s">
+        <v>77</v>
+      </c>
+      <c r="E91" s="23"/>
+      <c r="F91" s="23"/>
       <c r="G91" s="19"/>
     </row>
     <row r="92" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A92" s="39"/>
       <c r="B92" s="36"/>
-      <c r="C92" s="35" t="s">
-        <v>47</v>
-      </c>
-      <c r="D92" s="15" t="s">
-        <v>78</v>
-      </c>
-      <c r="E92" s="23"/>
-      <c r="F92" s="23"/>
+      <c r="C92" s="36"/>
+      <c r="D92" s="15"/>
+      <c r="E92" s="15"/>
+      <c r="F92" s="15"/>
       <c r="G92" s="19"/>
     </row>
     <row r="93" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A93" s="39"/>
       <c r="B93" s="36"/>
-      <c r="C93" s="36"/>
-      <c r="D93" s="15"/>
-      <c r="E93" s="15"/>
-      <c r="F93" s="15"/>
+      <c r="C93" s="35" t="s">
+        <v>49</v>
+      </c>
+      <c r="D93" s="15" t="s">
+        <v>125</v>
+      </c>
+      <c r="E93" s="23"/>
+      <c r="F93" s="23"/>
       <c r="G93" s="19"/>
     </row>
     <row r="94" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A94" s="39"/>
       <c r="B94" s="36"/>
-      <c r="C94" s="35" t="s">
-        <v>48</v>
-      </c>
+      <c r="C94" s="36"/>
       <c r="D94" s="15" t="s">
-        <v>77</v>
+        <v>126</v>
       </c>
       <c r="E94" s="23"/>
       <c r="F94" s="23"/>
@@ -4297,74 +4358,76 @@
       <c r="A95" s="39"/>
       <c r="B95" s="36"/>
       <c r="C95" s="36"/>
-      <c r="D95" s="15"/>
-      <c r="E95" s="15"/>
-      <c r="F95" s="15"/>
+      <c r="D95" s="15" t="s">
+        <v>127</v>
+      </c>
+      <c r="E95" s="23"/>
+      <c r="F95" s="23"/>
       <c r="G95" s="19"/>
     </row>
     <row r="96" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A96" s="39"/>
       <c r="B96" s="36"/>
-      <c r="C96" s="35" t="s">
-        <v>49</v>
-      </c>
-      <c r="D96" s="15" t="s">
-        <v>125</v>
-      </c>
-      <c r="E96" s="23"/>
-      <c r="F96" s="23"/>
+      <c r="C96" s="36"/>
+      <c r="D96" s="15"/>
+      <c r="E96" s="15"/>
+      <c r="F96" s="15"/>
       <c r="G96" s="19"/>
     </row>
     <row r="97" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A97" s="39"/>
       <c r="B97" s="36"/>
       <c r="C97" s="36"/>
-      <c r="D97" s="15" t="s">
-        <v>126</v>
-      </c>
-      <c r="E97" s="23"/>
-      <c r="F97" s="23"/>
+      <c r="D97" s="15"/>
+      <c r="E97" s="15"/>
+      <c r="F97" s="15"/>
       <c r="G97" s="19"/>
     </row>
-    <row r="98" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="98" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A98" s="39"/>
-      <c r="B98" s="36"/>
-      <c r="C98" s="36"/>
+      <c r="B98" s="35" t="s">
+        <v>21</v>
+      </c>
+      <c r="C98" s="35" t="s">
+        <v>50</v>
+      </c>
       <c r="D98" s="15" t="s">
-        <v>127</v>
+        <v>70</v>
       </c>
       <c r="E98" s="23"/>
       <c r="F98" s="23"/>
       <c r="G98" s="19"/>
     </row>
-    <row r="99" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="99" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A99" s="39"/>
       <c r="B99" s="36"/>
       <c r="C99" s="36"/>
-      <c r="D99" s="15"/>
-      <c r="E99" s="15"/>
-      <c r="F99" s="15"/>
+      <c r="D99" s="15" t="s">
+        <v>71</v>
+      </c>
+      <c r="E99" s="23"/>
+      <c r="F99" s="23"/>
       <c r="G99" s="19"/>
     </row>
-    <row r="100" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="100" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A100" s="39"/>
       <c r="B100" s="36"/>
       <c r="C100" s="36"/>
-      <c r="D100" s="15"/>
-      <c r="E100" s="15"/>
-      <c r="F100" s="15"/>
+      <c r="D100" s="15" t="s">
+        <v>83</v>
+      </c>
+      <c r="E100" s="23"/>
+      <c r="F100" s="23"/>
       <c r="G100" s="19"/>
     </row>
     <row r="101" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A101" s="39"/>
-      <c r="B101" s="35" t="s">
-        <v>21</v>
-      </c>
+      <c r="B101" s="36"/>
       <c r="C101" s="35" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D101" s="15" t="s">
-        <v>70</v>
+        <v>116</v>
       </c>
       <c r="E101" s="23"/>
       <c r="F101" s="23"/>
@@ -4375,7 +4438,7 @@
       <c r="B102" s="36"/>
       <c r="C102" s="36"/>
       <c r="D102" s="15" t="s">
-        <v>71</v>
+        <v>117</v>
       </c>
       <c r="E102" s="23"/>
       <c r="F102" s="23"/>
@@ -4386,7 +4449,7 @@
       <c r="B103" s="36"/>
       <c r="C103" s="36"/>
       <c r="D103" s="15" t="s">
-        <v>83</v>
+        <v>118</v>
       </c>
       <c r="E103" s="23"/>
       <c r="F103" s="23"/>
@@ -4395,11 +4458,9 @@
     <row r="104" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A104" s="39"/>
       <c r="B104" s="36"/>
-      <c r="C104" s="35" t="s">
-        <v>51</v>
-      </c>
+      <c r="C104" s="36"/>
       <c r="D104" s="15" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="E104" s="23"/>
       <c r="F104" s="23"/>
@@ -4408,9 +4469,11 @@
     <row r="105" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A105" s="39"/>
       <c r="B105" s="36"/>
-      <c r="C105" s="36"/>
+      <c r="C105" s="35" t="s">
+        <v>52</v>
+      </c>
       <c r="D105" s="15" t="s">
-        <v>117</v>
+        <v>122</v>
       </c>
       <c r="E105" s="23"/>
       <c r="F105" s="23"/>
@@ -4420,19 +4483,19 @@
       <c r="A106" s="39"/>
       <c r="B106" s="36"/>
       <c r="C106" s="36"/>
-      <c r="D106" s="15" t="s">
-        <v>118</v>
-      </c>
-      <c r="E106" s="23"/>
-      <c r="F106" s="23"/>
+      <c r="D106" s="15"/>
+      <c r="E106" s="15"/>
+      <c r="F106" s="15"/>
       <c r="G106" s="19"/>
     </row>
     <row r="107" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A107" s="39"/>
       <c r="B107" s="36"/>
-      <c r="C107" s="36"/>
+      <c r="C107" s="13" t="s">
+        <v>53</v>
+      </c>
       <c r="D107" s="15" t="s">
-        <v>119</v>
+        <v>86</v>
       </c>
       <c r="E107" s="23"/>
       <c r="F107" s="23"/>
@@ -4440,12 +4503,14 @@
     </row>
     <row r="108" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A108" s="39"/>
-      <c r="B108" s="36"/>
+      <c r="B108" s="35" t="s">
+        <v>22</v>
+      </c>
       <c r="C108" s="35" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="D108" s="15" t="s">
-        <v>122</v>
+        <v>92</v>
       </c>
       <c r="E108" s="23"/>
       <c r="F108" s="23"/>
@@ -4454,20 +4519,22 @@
     <row r="109" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A109" s="39"/>
       <c r="B109" s="36"/>
-      <c r="C109" s="36"/>
-      <c r="D109" s="15"/>
-      <c r="E109" s="15"/>
-      <c r="F109" s="15"/>
+      <c r="C109" s="37"/>
+      <c r="D109" s="15" t="s">
+        <v>93</v>
+      </c>
+      <c r="E109" s="23"/>
+      <c r="F109" s="23"/>
       <c r="G109" s="19"/>
     </row>
     <row r="110" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A110" s="39"/>
       <c r="B110" s="36"/>
-      <c r="C110" s="13" t="s">
-        <v>53</v>
+      <c r="C110" s="35" t="s">
+        <v>55</v>
       </c>
       <c r="D110" s="15" t="s">
-        <v>86</v>
+        <v>102</v>
       </c>
       <c r="E110" s="23"/>
       <c r="F110" s="23"/>
@@ -4475,499 +4542,489 @@
     </row>
     <row r="111" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A111" s="39"/>
-      <c r="B111" s="35" t="s">
-        <v>22</v>
-      </c>
-      <c r="C111" s="35" t="s">
-        <v>54</v>
-      </c>
-      <c r="D111" s="15" t="s">
-        <v>92</v>
-      </c>
-      <c r="E111" s="23"/>
-      <c r="F111" s="23"/>
+      <c r="B111" s="37"/>
+      <c r="C111" s="37"/>
+      <c r="D111" s="15"/>
+      <c r="E111" s="15"/>
+      <c r="F111" s="15"/>
       <c r="G111" s="19"/>
     </row>
     <row r="112" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A112" s="39"/>
-      <c r="B112" s="36"/>
-      <c r="C112" s="37"/>
-      <c r="D112" s="15" t="s">
-        <v>93</v>
-      </c>
-      <c r="E112" s="23"/>
-      <c r="F112" s="23"/>
+      <c r="B112" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="C112" s="11"/>
+      <c r="D112" s="15"/>
+      <c r="E112" s="15"/>
+      <c r="F112" s="15"/>
       <c r="G112" s="19"/>
     </row>
     <row r="113" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A113" s="39"/>
-      <c r="B113" s="36"/>
-      <c r="C113" s="35" t="s">
-        <v>55</v>
-      </c>
-      <c r="D113" s="15" t="s">
-        <v>102</v>
-      </c>
-      <c r="E113" s="23"/>
-      <c r="F113" s="23"/>
+      <c r="B113" s="11"/>
+      <c r="C113" s="11"/>
+      <c r="D113" s="15"/>
+      <c r="E113" s="15"/>
+      <c r="F113" s="15"/>
       <c r="G113" s="19"/>
     </row>
     <row r="114" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A114" s="39"/>
-      <c r="B114" s="37"/>
-      <c r="C114" s="37"/>
+      <c r="B114" s="11"/>
+      <c r="C114" s="11"/>
       <c r="D114" s="15"/>
       <c r="E114" s="15"/>
       <c r="F114" s="15"/>
       <c r="G114" s="19"/>
     </row>
     <row r="115" spans="1:8" x14ac:dyDescent="0.45">
-      <c r="A115" s="39"/>
-      <c r="B115" s="10" t="s">
-        <v>23</v>
-      </c>
-      <c r="C115" s="11"/>
+      <c r="A115" s="40"/>
+      <c r="B115" s="12"/>
+      <c r="C115" s="12"/>
       <c r="D115" s="15"/>
       <c r="E115" s="15"/>
       <c r="F115" s="15"/>
       <c r="G115" s="19"/>
     </row>
     <row r="116" spans="1:8" x14ac:dyDescent="0.45">
-      <c r="A116" s="39"/>
-      <c r="B116" s="11"/>
-      <c r="C116" s="11"/>
-      <c r="D116" s="15"/>
-      <c r="E116" s="15"/>
-      <c r="F116" s="15"/>
+      <c r="A116" s="38" t="s">
+        <v>140</v>
+      </c>
+      <c r="B116" s="43" t="s">
+        <v>141</v>
+      </c>
+      <c r="C116" s="28"/>
+      <c r="D116" s="19"/>
+      <c r="E116" s="19"/>
+      <c r="F116" s="19"/>
       <c r="G116" s="19"/>
     </row>
     <row r="117" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A117" s="39"/>
-      <c r="B117" s="11"/>
-      <c r="C117" s="11"/>
-      <c r="D117" s="15"/>
-      <c r="E117" s="15"/>
-      <c r="F117" s="15"/>
+      <c r="B117" s="41"/>
+      <c r="C117" s="28"/>
+      <c r="D117" s="19"/>
+      <c r="E117" s="19"/>
+      <c r="F117" s="19"/>
       <c r="G117" s="19"/>
     </row>
     <row r="118" spans="1:8" x14ac:dyDescent="0.45">
-      <c r="A118" s="40"/>
-      <c r="B118" s="12"/>
-      <c r="C118" s="12"/>
-      <c r="D118" s="15"/>
-      <c r="E118" s="15"/>
-      <c r="F118" s="15"/>
+      <c r="A118" s="39"/>
+      <c r="B118" s="42"/>
+      <c r="C118" s="28"/>
+      <c r="D118" s="19"/>
+      <c r="E118" s="19"/>
+      <c r="F118" s="19"/>
       <c r="G118" s="19"/>
     </row>
     <row r="119" spans="1:8" x14ac:dyDescent="0.45">
-      <c r="A119" s="38" t="s">
-        <v>140</v>
-      </c>
+      <c r="A119" s="39"/>
       <c r="B119" s="43" t="s">
-        <v>141</v>
-      </c>
-      <c r="C119" s="28"/>
+        <v>142</v>
+      </c>
+      <c r="C119" s="28" t="s">
+        <v>146</v>
+      </c>
       <c r="D119" s="19"/>
       <c r="E119" s="19"/>
       <c r="F119" s="19"/>
       <c r="G119" s="19"/>
+      <c r="H119" s="9" t="s">
+        <v>179</v>
+      </c>
     </row>
     <row r="120" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A120" s="39"/>
       <c r="B120" s="41"/>
-      <c r="C120" s="28"/>
-      <c r="D120" s="19"/>
+      <c r="C120" s="28" t="s">
+        <v>145</v>
+      </c>
+      <c r="D120" s="19" t="s">
+        <v>185</v>
+      </c>
       <c r="E120" s="19"/>
-      <c r="F120" s="19"/>
-      <c r="G120" s="19"/>
+      <c r="F120" s="16" t="s">
+        <v>190</v>
+      </c>
+      <c r="G120" s="19" t="s">
+        <v>188</v>
+      </c>
     </row>
     <row r="121" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A121" s="39"/>
-      <c r="B121" s="42"/>
+      <c r="B121" s="41"/>
       <c r="C121" s="28"/>
-      <c r="D121" s="19"/>
+      <c r="D121" s="19" t="s">
+        <v>186</v>
+      </c>
       <c r="E121" s="19"/>
-      <c r="F121" s="19"/>
-      <c r="G121" s="19"/>
+      <c r="F121" s="16" t="s">
+        <v>190</v>
+      </c>
+      <c r="G121" s="19" t="s">
+        <v>188</v>
+      </c>
     </row>
     <row r="122" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A122" s="39"/>
-      <c r="B122" s="43" t="s">
-        <v>142</v>
-      </c>
-      <c r="C122" s="28" t="s">
-        <v>146</v>
-      </c>
-      <c r="D122" s="19"/>
+      <c r="B122" s="41"/>
+      <c r="C122" s="28"/>
+      <c r="D122" s="19" t="s">
+        <v>187</v>
+      </c>
       <c r="E122" s="19"/>
-      <c r="F122" s="19"/>
-      <c r="G122" s="19"/>
-      <c r="H122" s="9" t="s">
-        <v>179</v>
+      <c r="F122" s="16" t="s">
+        <v>190</v>
+      </c>
+      <c r="G122" s="19" t="s">
+        <v>189</v>
       </c>
     </row>
     <row r="123" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A123" s="39"/>
       <c r="B123" s="41"/>
       <c r="C123" s="28" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="D123" s="19" t="s">
-        <v>185</v>
+        <v>178</v>
       </c>
       <c r="E123" s="19"/>
       <c r="F123" s="16" t="s">
         <v>190</v>
       </c>
       <c r="G123" s="19" t="s">
-        <v>188</v>
+        <v>183</v>
       </c>
     </row>
     <row r="124" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A124" s="39"/>
       <c r="B124" s="41"/>
-      <c r="C124" s="28"/>
+      <c r="C124" s="28" t="s">
+        <v>148</v>
+      </c>
       <c r="D124" s="19" t="s">
-        <v>186</v>
+        <v>176</v>
       </c>
       <c r="E124" s="19"/>
-      <c r="F124" s="16" t="s">
-        <v>190</v>
-      </c>
+      <c r="F124" s="19"/>
       <c r="G124" s="19" t="s">
-        <v>188</v>
+        <v>177</v>
       </c>
     </row>
     <row r="125" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A125" s="39"/>
       <c r="B125" s="41"/>
-      <c r="C125" s="28"/>
+      <c r="C125" s="28" t="s">
+        <v>149</v>
+      </c>
       <c r="D125" s="19" t="s">
-        <v>187</v>
+        <v>174</v>
       </c>
       <c r="E125" s="19"/>
       <c r="F125" s="16" t="s">
         <v>190</v>
       </c>
       <c r="G125" s="19" t="s">
-        <v>189</v>
+        <v>177</v>
       </c>
     </row>
     <row r="126" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A126" s="39"/>
       <c r="B126" s="41"/>
       <c r="C126" s="28" t="s">
-        <v>147</v>
+        <v>173</v>
       </c>
       <c r="D126" s="19" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="E126" s="19"/>
-      <c r="F126" s="16" t="s">
-        <v>190</v>
-      </c>
-      <c r="G126" s="19" t="s">
-        <v>183</v>
-      </c>
+      <c r="F126" s="19"/>
+      <c r="G126" s="19"/>
     </row>
     <row r="127" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A127" s="39"/>
       <c r="B127" s="41"/>
-      <c r="C127" s="28" t="s">
-        <v>148</v>
-      </c>
-      <c r="D127" s="19" t="s">
-        <v>176</v>
-      </c>
+      <c r="C127" s="28"/>
+      <c r="D127" s="19"/>
       <c r="E127" s="19"/>
       <c r="F127" s="19"/>
-      <c r="G127" s="19" t="s">
-        <v>177</v>
-      </c>
+      <c r="G127" s="19"/>
     </row>
     <row r="128" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A128" s="39"/>
       <c r="B128" s="41"/>
-      <c r="C128" s="28" t="s">
-        <v>149</v>
-      </c>
-      <c r="D128" s="19" t="s">
-        <v>174</v>
-      </c>
+      <c r="C128" s="28"/>
+      <c r="D128" s="19"/>
       <c r="E128" s="19"/>
-      <c r="F128" s="16" t="s">
-        <v>190</v>
-      </c>
-      <c r="G128" s="19" t="s">
-        <v>177</v>
-      </c>
+      <c r="F128" s="19"/>
+      <c r="G128" s="19"/>
     </row>
     <row r="129" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A129" s="39"/>
       <c r="B129" s="41"/>
-      <c r="C129" s="28" t="s">
-        <v>173</v>
-      </c>
-      <c r="D129" s="19" t="s">
-        <v>175</v>
-      </c>
+      <c r="C129" s="28"/>
+      <c r="D129" s="19"/>
       <c r="E129" s="19"/>
       <c r="F129" s="19"/>
       <c r="G129" s="19"/>
     </row>
-    <row r="130" spans="1:8" x14ac:dyDescent="0.45">
-      <c r="A130" s="39"/>
-      <c r="B130" s="41"/>
-      <c r="C130" s="28"/>
-      <c r="D130" s="19"/>
-      <c r="E130" s="19"/>
-      <c r="F130" s="19"/>
-      <c r="G130" s="19"/>
+    <row r="130" spans="1:8" ht="17.5" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="A130" s="47"/>
+      <c r="B130" s="48"/>
+      <c r="C130" s="31"/>
+      <c r="D130" s="32"/>
+      <c r="E130" s="33"/>
+      <c r="F130" s="33"/>
+      <c r="G130" s="32"/>
     </row>
     <row r="131" spans="1:8" x14ac:dyDescent="0.45">
-      <c r="A131" s="39"/>
-      <c r="B131" s="41"/>
-      <c r="C131" s="28"/>
-      <c r="D131" s="19"/>
-      <c r="E131" s="19"/>
-      <c r="F131" s="19"/>
-      <c r="G131" s="19"/>
+      <c r="A131" s="39" t="s">
+        <v>150</v>
+      </c>
+      <c r="B131" s="41" t="s">
+        <v>151</v>
+      </c>
+      <c r="C131" s="45" t="s">
+        <v>153</v>
+      </c>
+      <c r="D131" s="30" t="s">
+        <v>164</v>
+      </c>
+      <c r="E131" s="14" t="s">
+        <v>168</v>
+      </c>
+      <c r="F131" s="14"/>
+      <c r="G131" s="20" t="s">
+        <v>156</v>
+      </c>
+      <c r="H131" s="9" t="s">
+        <v>169</v>
+      </c>
     </row>
     <row r="132" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A132" s="39"/>
       <c r="B132" s="41"/>
-      <c r="C132" s="28"/>
-      <c r="D132" s="19"/>
-      <c r="E132" s="19"/>
-      <c r="F132" s="19"/>
-      <c r="G132" s="19"/>
-    </row>
-    <row r="133" spans="1:8" ht="17.5" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A133" s="47"/>
-      <c r="B133" s="48"/>
-      <c r="C133" s="31"/>
-      <c r="D133" s="32"/>
-      <c r="E133" s="33"/>
-      <c r="F133" s="33"/>
-      <c r="G133" s="32"/>
+      <c r="C132" s="45"/>
+      <c r="D132" s="17" t="s">
+        <v>161</v>
+      </c>
+      <c r="E132" s="16" t="s">
+        <v>168</v>
+      </c>
+      <c r="F132" s="16"/>
+      <c r="G132" s="19" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="133" spans="1:8" x14ac:dyDescent="0.45">
+      <c r="A133" s="39"/>
+      <c r="B133" s="41"/>
+      <c r="C133" s="45"/>
+      <c r="D133" s="17" t="s">
+        <v>162</v>
+      </c>
+      <c r="E133" s="16" t="s">
+        <v>168</v>
+      </c>
+      <c r="F133" s="16"/>
+      <c r="G133" s="19" t="s">
+        <v>156</v>
+      </c>
     </row>
     <row r="134" spans="1:8" x14ac:dyDescent="0.45">
-      <c r="A134" s="39" t="s">
-        <v>150</v>
-      </c>
-      <c r="B134" s="41" t="s">
-        <v>151</v>
-      </c>
-      <c r="C134" s="45" t="s">
-        <v>153</v>
-      </c>
-      <c r="D134" s="30" t="s">
-        <v>164</v>
-      </c>
-      <c r="E134" s="14" t="s">
+      <c r="A134" s="39"/>
+      <c r="B134" s="41"/>
+      <c r="C134" s="46"/>
+      <c r="D134" s="17" t="s">
+        <v>163</v>
+      </c>
+      <c r="E134" s="16" t="s">
         <v>168</v>
       </c>
-      <c r="F134" s="14"/>
-      <c r="G134" s="20" t="s">
+      <c r="F134" s="16"/>
+      <c r="G134" s="19" t="s">
         <v>156</v>
-      </c>
-      <c r="H134" s="9" t="s">
-        <v>169</v>
       </c>
     </row>
     <row r="135" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A135" s="39"/>
       <c r="B135" s="41"/>
-      <c r="C135" s="45"/>
+      <c r="C135" s="28" t="s">
+        <v>154</v>
+      </c>
       <c r="D135" s="17" t="s">
-        <v>161</v>
+        <v>155</v>
       </c>
       <c r="E135" s="16" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="F135" s="16"/>
-      <c r="G135" s="19" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="136" spans="1:8" x14ac:dyDescent="0.45">
+      <c r="G135" s="19"/>
+    </row>
+    <row r="136" spans="1:8" ht="102" x14ac:dyDescent="0.45">
       <c r="A136" s="39"/>
       <c r="B136" s="41"/>
-      <c r="C136" s="45"/>
+      <c r="C136" s="44" t="s">
+        <v>165</v>
+      </c>
       <c r="D136" s="17" t="s">
-        <v>162</v>
+        <v>196</v>
       </c>
       <c r="E136" s="16" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="F136" s="16"/>
-      <c r="G136" s="19" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="137" spans="1:8" x14ac:dyDescent="0.45">
+      <c r="G136" s="17" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="137" spans="1:8" ht="51" x14ac:dyDescent="0.45">
       <c r="A137" s="39"/>
       <c r="B137" s="41"/>
-      <c r="C137" s="46"/>
+      <c r="C137" s="45"/>
       <c r="D137" s="17" t="s">
-        <v>163</v>
+        <v>201</v>
       </c>
       <c r="E137" s="16" t="s">
-        <v>168</v>
+        <v>132</v>
       </c>
       <c r="F137" s="16"/>
-      <c r="G137" s="19" t="s">
-        <v>156</v>
+      <c r="G137" s="17" t="s">
+        <v>202</v>
       </c>
     </row>
     <row r="138" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A138" s="39"/>
       <c r="B138" s="41"/>
-      <c r="C138" s="28" t="s">
-        <v>154</v>
-      </c>
+      <c r="C138" s="45"/>
       <c r="D138" s="17" t="s">
-        <v>155</v>
+        <v>198</v>
       </c>
       <c r="E138" s="16" t="s">
-        <v>167</v>
+        <v>131</v>
       </c>
       <c r="F138" s="16"/>
-      <c r="G138" s="19"/>
-    </row>
-    <row r="139" spans="1:8" ht="102" x14ac:dyDescent="0.45">
+      <c r="G138" s="19" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="139" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A139" s="39"/>
       <c r="B139" s="41"/>
-      <c r="C139" s="44" t="s">
-        <v>165</v>
-      </c>
+      <c r="C139" s="45"/>
       <c r="D139" s="17" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="E139" s="16" t="s">
-        <v>167</v>
+        <v>131</v>
       </c>
       <c r="F139" s="16"/>
-      <c r="G139" s="17" t="s">
-        <v>203</v>
-      </c>
-    </row>
-    <row r="140" spans="1:8" ht="51" x14ac:dyDescent="0.45">
+      <c r="G139" s="19" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="140" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A140" s="39"/>
       <c r="B140" s="41"/>
-      <c r="C140" s="45"/>
+      <c r="C140" s="46"/>
       <c r="D140" s="17" t="s">
-        <v>201</v>
-      </c>
-      <c r="E140" s="16" t="s">
-        <v>132</v>
-      </c>
+        <v>194</v>
+      </c>
+      <c r="E140" s="16"/>
       <c r="F140" s="16"/>
-      <c r="G140" s="17" t="s">
-        <v>202</v>
+      <c r="G140" s="19" t="s">
+        <v>200</v>
       </c>
     </row>
     <row r="141" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A141" s="39"/>
       <c r="B141" s="41"/>
-      <c r="C141" s="45"/>
+      <c r="C141" s="44" t="s">
+        <v>166</v>
+      </c>
       <c r="D141" s="17" t="s">
-        <v>198</v>
-      </c>
-      <c r="E141" s="16" t="s">
-        <v>131</v>
-      </c>
+        <v>157</v>
+      </c>
+      <c r="E141" s="16"/>
       <c r="F141" s="16"/>
-      <c r="G141" s="19" t="s">
-        <v>199</v>
-      </c>
+      <c r="G141" s="19"/>
     </row>
     <row r="142" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A142" s="39"/>
       <c r="B142" s="41"/>
       <c r="C142" s="45"/>
       <c r="D142" s="17" t="s">
-        <v>195</v>
-      </c>
-      <c r="E142" s="16" t="s">
-        <v>131</v>
-      </c>
+        <v>160</v>
+      </c>
+      <c r="E142" s="16"/>
       <c r="F142" s="16"/>
-      <c r="G142" s="19" t="s">
-        <v>197</v>
-      </c>
+      <c r="G142" s="19"/>
     </row>
     <row r="143" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A143" s="39"/>
       <c r="B143" s="41"/>
-      <c r="C143" s="46"/>
+      <c r="C143" s="45"/>
       <c r="D143" s="17" t="s">
-        <v>194</v>
+        <v>159</v>
       </c>
       <c r="E143" s="16"/>
       <c r="F143" s="16"/>
-      <c r="G143" s="19" t="s">
-        <v>200</v>
-      </c>
+      <c r="G143" s="19"/>
     </row>
     <row r="144" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A144" s="39"/>
       <c r="B144" s="41"/>
-      <c r="C144" s="44" t="s">
-        <v>166</v>
-      </c>
-      <c r="D144" s="17" t="s">
-        <v>157</v>
+      <c r="C144" s="46"/>
+      <c r="D144" s="19" t="s">
+        <v>158</v>
       </c>
       <c r="E144" s="16"/>
       <c r="F144" s="16"/>
       <c r="G144" s="19"/>
     </row>
-    <row r="145" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="145" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A145" s="39"/>
       <c r="B145" s="41"/>
-      <c r="C145" s="45"/>
-      <c r="D145" s="17" t="s">
-        <v>160</v>
-      </c>
+      <c r="C145" s="28" t="s">
+        <v>152</v>
+      </c>
+      <c r="D145" s="19"/>
       <c r="E145" s="16"/>
       <c r="F145" s="16"/>
       <c r="G145" s="19"/>
     </row>
-    <row r="146" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="146" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A146" s="39"/>
-      <c r="B146" s="41"/>
-      <c r="C146" s="45"/>
-      <c r="D146" s="17" t="s">
-        <v>159</v>
-      </c>
+      <c r="B146" s="42"/>
+      <c r="C146" s="28"/>
+      <c r="D146" s="19"/>
       <c r="E146" s="16"/>
       <c r="F146" s="16"/>
       <c r="G146" s="19"/>
     </row>
-    <row r="147" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="147" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A147" s="39"/>
-      <c r="B147" s="41"/>
-      <c r="C147" s="46"/>
-      <c r="D147" s="19" t="s">
-        <v>158</v>
-      </c>
+      <c r="B147" s="43" t="s">
+        <v>170</v>
+      </c>
+      <c r="C147" s="28"/>
+      <c r="D147" s="19"/>
       <c r="E147" s="16"/>
       <c r="F147" s="16"/>
       <c r="G147" s="19"/>
     </row>
-    <row r="148" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="148" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A148" s="39"/>
       <c r="B148" s="41"/>
-      <c r="C148" s="28" t="s">
-        <v>152</v>
-      </c>
+      <c r="C148" s="28"/>
       <c r="D148" s="19"/>
       <c r="E148" s="16"/>
       <c r="F148" s="16"/>
       <c r="G148" s="19"/>
     </row>
-    <row r="149" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="149" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A149" s="39"/>
       <c r="B149" s="42"/>
       <c r="C149" s="28"/>
@@ -4976,10 +5033,10 @@
       <c r="F149" s="16"/>
       <c r="G149" s="19"/>
     </row>
-    <row r="150" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="150" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A150" s="39"/>
-      <c r="B150" s="43" t="s">
-        <v>170</v>
+      <c r="B150" s="29" t="s">
+        <v>171</v>
       </c>
       <c r="C150" s="28"/>
       <c r="D150" s="19"/>
@@ -4987,201 +5044,1731 @@
       <c r="F150" s="16"/>
       <c r="G150" s="19"/>
     </row>
-    <row r="151" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="151" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A151" s="39"/>
-      <c r="B151" s="41"/>
+      <c r="B151" s="43" t="s">
+        <v>172</v>
+      </c>
       <c r="C151" s="28"/>
       <c r="D151" s="19"/>
       <c r="E151" s="16"/>
       <c r="F151" s="16"/>
       <c r="G151" s="19"/>
     </row>
-    <row r="152" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="152" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A152" s="39"/>
-      <c r="B152" s="42"/>
-      <c r="C152" s="28"/>
+      <c r="B152" s="41"/>
+      <c r="C152" s="28" t="s">
+        <v>180</v>
+      </c>
       <c r="D152" s="19"/>
       <c r="E152" s="16"/>
       <c r="F152" s="16"/>
       <c r="G152" s="19"/>
     </row>
-    <row r="153" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="153" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A153" s="39"/>
-      <c r="B153" s="29" t="s">
-        <v>171</v>
-      </c>
-      <c r="C153" s="28"/>
+      <c r="B153" s="41"/>
+      <c r="C153" s="28" t="s">
+        <v>182</v>
+      </c>
       <c r="D153" s="19"/>
       <c r="E153" s="16"/>
       <c r="F153" s="16"/>
-      <c r="G153" s="19"/>
-    </row>
-    <row r="154" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="G153" s="19" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="154" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A154" s="39"/>
-      <c r="B154" s="43" t="s">
-        <v>172</v>
-      </c>
-      <c r="C154" s="28"/>
+      <c r="B154" s="41"/>
+      <c r="C154" s="28" t="s">
+        <v>181</v>
+      </c>
       <c r="D154" s="19"/>
       <c r="E154" s="16"/>
       <c r="F154" s="16"/>
       <c r="G154" s="19"/>
     </row>
-    <row r="155" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="155" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A155" s="39"/>
       <c r="B155" s="41"/>
-      <c r="C155" s="28" t="s">
-        <v>180</v>
-      </c>
+      <c r="C155" s="28"/>
       <c r="D155" s="19"/>
       <c r="E155" s="16"/>
       <c r="F155" s="16"/>
       <c r="G155" s="19"/>
     </row>
-    <row r="156" spans="1:7" x14ac:dyDescent="0.45">
+    <row r="156" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A156" s="39"/>
       <c r="B156" s="41"/>
-      <c r="C156" s="28" t="s">
-        <v>182</v>
-      </c>
+      <c r="C156" s="28"/>
       <c r="D156" s="19"/>
       <c r="E156" s="16"/>
       <c r="F156" s="16"/>
-      <c r="G156" s="19" t="s">
-        <v>183</v>
-      </c>
-    </row>
-    <row r="157" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="G156" s="19"/>
+    </row>
+    <row r="157" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A157" s="39"/>
       <c r="B157" s="41"/>
-      <c r="C157" s="28" t="s">
-        <v>181</v>
-      </c>
+      <c r="C157" s="28"/>
       <c r="D157" s="19"/>
       <c r="E157" s="16"/>
       <c r="F157" s="16"/>
       <c r="G157" s="19"/>
     </row>
-    <row r="158" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A158" s="39"/>
-      <c r="B158" s="41"/>
+    <row r="158" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A158" s="40"/>
+      <c r="B158" s="42"/>
       <c r="C158" s="28"/>
       <c r="D158" s="19"/>
       <c r="E158" s="16"/>
       <c r="F158" s="16"/>
       <c r="G158" s="19"/>
     </row>
-    <row r="159" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A159" s="39"/>
-      <c r="B159" s="41"/>
-      <c r="C159" s="28"/>
-      <c r="D159" s="19"/>
-      <c r="E159" s="16"/>
-      <c r="F159" s="16"/>
-      <c r="G159" s="19"/>
-    </row>
-    <row r="160" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A160" s="39"/>
-      <c r="B160" s="41"/>
-      <c r="C160" s="28"/>
-      <c r="D160" s="19"/>
-      <c r="E160" s="16"/>
-      <c r="F160" s="16"/>
-      <c r="G160" s="19"/>
-    </row>
-    <row r="161" spans="1:9" x14ac:dyDescent="0.45">
-      <c r="A161" s="40"/>
-      <c r="B161" s="42"/>
-      <c r="C161" s="28"/>
-      <c r="D161" s="19"/>
-      <c r="E161" s="16"/>
-      <c r="F161" s="16"/>
-      <c r="G161" s="19"/>
-    </row>
-    <row r="162" spans="1:9" x14ac:dyDescent="0.45">
-      <c r="B162" t="s">
+    <row r="159" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="B159" t="s">
         <v>144</v>
       </c>
-      <c r="C162" t="s">
+      <c r="C159" t="s">
         <v>143</v>
       </c>
     </row>
-    <row r="163" spans="1:9" x14ac:dyDescent="0.45">
-      <c r="I163" s="7"/>
-    </row>
-    <row r="164" spans="1:9" x14ac:dyDescent="0.45">
-      <c r="C164" t="s">
+    <row r="160" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="I160" s="7"/>
+    </row>
+    <row r="161" spans="3:9" x14ac:dyDescent="0.45">
+      <c r="C161" t="s">
         <v>193</v>
       </c>
-      <c r="I164" s="8"/>
-    </row>
-    <row r="165" spans="1:9" x14ac:dyDescent="0.45">
-      <c r="I165" s="8"/>
+      <c r="I161" s="8"/>
+    </row>
+    <row r="162" spans="3:9" x14ac:dyDescent="0.45">
+      <c r="I162" s="8"/>
     </row>
   </sheetData>
-  <autoFilter ref="A4:G119" xr:uid="{34DC90E1-7112-4806-ADC5-98CA8498E977}"/>
-  <mergeCells count="58">
-    <mergeCell ref="C9:C10"/>
-    <mergeCell ref="C16:C18"/>
-    <mergeCell ref="C21:C24"/>
-    <mergeCell ref="C25:C28"/>
-    <mergeCell ref="B150:B152"/>
-    <mergeCell ref="C92:C93"/>
-    <mergeCell ref="C94:C95"/>
-    <mergeCell ref="C96:C100"/>
+  <autoFilter ref="A4:G116" xr:uid="{34DC90E1-7112-4806-ADC5-98CA8498E977}"/>
+  <mergeCells count="56">
+    <mergeCell ref="C8:C9"/>
+    <mergeCell ref="C13:C15"/>
+    <mergeCell ref="C18:C21"/>
+    <mergeCell ref="C22:C25"/>
+    <mergeCell ref="B147:B149"/>
+    <mergeCell ref="C89:C90"/>
+    <mergeCell ref="C91:C92"/>
+    <mergeCell ref="C93:C97"/>
+    <mergeCell ref="C105:C106"/>
+    <mergeCell ref="B66:B79"/>
+    <mergeCell ref="C66:C68"/>
+    <mergeCell ref="C69:C71"/>
+    <mergeCell ref="C72:C75"/>
+    <mergeCell ref="C76:C77"/>
+    <mergeCell ref="C78:C79"/>
+    <mergeCell ref="B80:B83"/>
+    <mergeCell ref="C80:C81"/>
+    <mergeCell ref="A116:A130"/>
+    <mergeCell ref="B119:B130"/>
+    <mergeCell ref="B116:B118"/>
+    <mergeCell ref="B108:B111"/>
     <mergeCell ref="C108:C109"/>
-    <mergeCell ref="B69:B82"/>
-    <mergeCell ref="C69:C71"/>
-    <mergeCell ref="C72:C74"/>
-    <mergeCell ref="C75:C78"/>
-    <mergeCell ref="C79:C80"/>
-    <mergeCell ref="C81:C82"/>
-    <mergeCell ref="B83:B86"/>
-    <mergeCell ref="C83:C84"/>
-    <mergeCell ref="A119:A133"/>
-    <mergeCell ref="B122:B133"/>
-    <mergeCell ref="B119:B121"/>
-    <mergeCell ref="B111:B114"/>
-    <mergeCell ref="C111:C112"/>
-    <mergeCell ref="C113:C114"/>
-    <mergeCell ref="A5:A118"/>
-    <mergeCell ref="B5:B12"/>
-    <mergeCell ref="C7:C8"/>
-    <mergeCell ref="C11:C12"/>
-    <mergeCell ref="B13:B28"/>
-    <mergeCell ref="C13:C15"/>
-    <mergeCell ref="B101:B110"/>
-    <mergeCell ref="C101:C103"/>
-    <mergeCell ref="C104:C107"/>
-    <mergeCell ref="B61:B68"/>
-    <mergeCell ref="C61:C62"/>
-    <mergeCell ref="C63:C68"/>
-    <mergeCell ref="B29:B60"/>
+    <mergeCell ref="C110:C111"/>
+    <mergeCell ref="A5:A115"/>
+    <mergeCell ref="B5:B11"/>
+    <mergeCell ref="C10:C11"/>
+    <mergeCell ref="B12:B25"/>
+    <mergeCell ref="B98:B107"/>
+    <mergeCell ref="C98:C100"/>
+    <mergeCell ref="C101:C104"/>
+    <mergeCell ref="B58:B65"/>
+    <mergeCell ref="C58:C59"/>
+    <mergeCell ref="C60:C65"/>
+    <mergeCell ref="B26:B57"/>
+    <mergeCell ref="C26:C28"/>
     <mergeCell ref="C29:C31"/>
-    <mergeCell ref="C32:C34"/>
-    <mergeCell ref="C35:C38"/>
-    <mergeCell ref="C39:C40"/>
-    <mergeCell ref="C41:C42"/>
+    <mergeCell ref="C32:C35"/>
+    <mergeCell ref="C36:C37"/>
+    <mergeCell ref="C38:C39"/>
+    <mergeCell ref="C40:C42"/>
     <mergeCell ref="C43:C45"/>
-    <mergeCell ref="C46:C48"/>
-    <mergeCell ref="C49:C50"/>
+    <mergeCell ref="C46:C47"/>
+    <mergeCell ref="C48:C50"/>
     <mergeCell ref="C51:C53"/>
-    <mergeCell ref="C54:C56"/>
-    <mergeCell ref="A134:A161"/>
-    <mergeCell ref="B134:B149"/>
-    <mergeCell ref="B154:B161"/>
-    <mergeCell ref="C144:C147"/>
-    <mergeCell ref="C134:C137"/>
-    <mergeCell ref="C139:C143"/>
-    <mergeCell ref="C85:C86"/>
-    <mergeCell ref="B87:B100"/>
-    <mergeCell ref="C87:C89"/>
-    <mergeCell ref="C90:C91"/>
-    <mergeCell ref="C57:C58"/>
-    <mergeCell ref="C59:C60"/>
+    <mergeCell ref="A131:A158"/>
+    <mergeCell ref="B131:B146"/>
+    <mergeCell ref="B151:B158"/>
+    <mergeCell ref="C141:C144"/>
+    <mergeCell ref="C131:C134"/>
+    <mergeCell ref="C136:C140"/>
+    <mergeCell ref="C82:C83"/>
+    <mergeCell ref="B84:B97"/>
+    <mergeCell ref="C84:C86"/>
+    <mergeCell ref="C87:C88"/>
+    <mergeCell ref="C54:C55"/>
+    <mergeCell ref="C56:C57"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8EFC0EAB-5103-4A10-AA81-95D4B4AEDD51}">
+  <sheetPr>
+    <tabColor theme="5" tint="0.59999389629810485"/>
+  </sheetPr>
+  <dimension ref="A1:I133"/>
+  <sheetFormatPr defaultRowHeight="17" x14ac:dyDescent="0.45"/>
+  <cols>
+    <col min="1" max="1" width="21.25" customWidth="1"/>
+    <col min="2" max="2" width="18.58203125" customWidth="1"/>
+    <col min="3" max="3" width="29.08203125" customWidth="1"/>
+    <col min="4" max="4" width="29.83203125" style="3" customWidth="1"/>
+    <col min="5" max="6" width="10.83203125" style="5" customWidth="1"/>
+    <col min="7" max="7" width="56.25" style="3" customWidth="1"/>
+    <col min="8" max="8" width="28.58203125" style="9" customWidth="1"/>
+    <col min="9" max="9" width="7.5" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.45">
+      <c r="D1"/>
+    </row>
+    <row r="2" spans="1:8" s="4" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A2" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="E2" s="22"/>
+      <c r="F2" s="22"/>
+      <c r="G2" s="27"/>
+      <c r="H2" s="34"/>
+    </row>
+    <row r="3" spans="1:8" ht="8.25" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="D3"/>
+    </row>
+    <row r="4" spans="1:8" ht="26.25" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A4" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>184</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.45">
+      <c r="A5" s="38" t="s">
+        <v>4</v>
+      </c>
+      <c r="B5" s="35" t="s">
+        <v>5</v>
+      </c>
+      <c r="C5" s="13"/>
+      <c r="D5" s="15" t="s">
+        <v>85</v>
+      </c>
+      <c r="E5" s="24"/>
+      <c r="F5" s="24"/>
+      <c r="G5" s="19"/>
+      <c r="H5" s="9" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.45">
+      <c r="A6" s="39"/>
+      <c r="B6" s="36"/>
+      <c r="C6" s="13" t="s">
+        <v>130</v>
+      </c>
+      <c r="D6" s="15" t="s">
+        <v>206</v>
+      </c>
+      <c r="E6" s="23"/>
+      <c r="F6" s="16"/>
+      <c r="G6" s="19"/>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.45">
+      <c r="A7" s="39"/>
+      <c r="B7" s="36"/>
+      <c r="C7" s="13" t="s">
+        <v>7</v>
+      </c>
+      <c r="D7" s="15" t="s">
+        <v>205</v>
+      </c>
+      <c r="E7" s="23"/>
+      <c r="F7" s="16"/>
+      <c r="G7" s="19"/>
+    </row>
+    <row r="8" spans="1:8" ht="34" x14ac:dyDescent="0.45">
+      <c r="A8" s="39"/>
+      <c r="B8" s="36"/>
+      <c r="C8" s="35" t="s">
+        <v>191</v>
+      </c>
+      <c r="D8" s="15" t="s">
+        <v>88</v>
+      </c>
+      <c r="E8" s="24"/>
+      <c r="F8" s="16"/>
+      <c r="G8" s="17" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.45">
+      <c r="A9" s="39"/>
+      <c r="B9" s="36"/>
+      <c r="C9" s="36"/>
+      <c r="D9" s="15"/>
+      <c r="E9" s="15"/>
+      <c r="F9" s="15"/>
+      <c r="G9" s="19"/>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.45">
+      <c r="A10" s="39"/>
+      <c r="B10" s="36"/>
+      <c r="C10" s="35" t="s">
+        <v>192</v>
+      </c>
+      <c r="D10" s="17" t="s">
+        <v>87</v>
+      </c>
+      <c r="E10" s="24"/>
+      <c r="F10" s="24"/>
+      <c r="G10" s="19"/>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.45">
+      <c r="A11" s="39"/>
+      <c r="B11" s="36"/>
+      <c r="C11" s="36"/>
+      <c r="D11" s="17"/>
+      <c r="E11" s="17"/>
+      <c r="F11" s="17"/>
+      <c r="G11" s="19"/>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.45">
+      <c r="A12" s="39"/>
+      <c r="B12" s="35" t="s">
+        <v>6</v>
+      </c>
+      <c r="C12" s="13" t="s">
+        <v>10</v>
+      </c>
+      <c r="D12" s="18" t="s">
+        <v>107</v>
+      </c>
+      <c r="E12" s="25"/>
+      <c r="F12" s="16"/>
+      <c r="G12" s="19"/>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.45">
+      <c r="A13" s="39"/>
+      <c r="B13" s="36"/>
+      <c r="C13" s="35" t="s">
+        <v>11</v>
+      </c>
+      <c r="D13" s="18" t="s">
+        <v>59</v>
+      </c>
+      <c r="E13" s="25"/>
+      <c r="F13" s="16"/>
+      <c r="G13" s="19"/>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.45">
+      <c r="A14" s="39"/>
+      <c r="B14" s="36"/>
+      <c r="C14" s="36"/>
+      <c r="D14" s="18" t="s">
+        <v>60</v>
+      </c>
+      <c r="E14" s="25"/>
+      <c r="F14" s="25"/>
+      <c r="G14" s="19"/>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.45">
+      <c r="A15" s="39"/>
+      <c r="B15" s="36"/>
+      <c r="C15" s="37"/>
+      <c r="D15" s="18"/>
+      <c r="E15" s="18"/>
+      <c r="F15" s="18"/>
+      <c r="G15" s="19"/>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.45">
+      <c r="A16" s="39"/>
+      <c r="B16" s="36"/>
+      <c r="C16" s="13" t="s">
+        <v>12</v>
+      </c>
+      <c r="D16" s="18" t="s">
+        <v>63</v>
+      </c>
+      <c r="E16" s="25"/>
+      <c r="F16" s="16"/>
+      <c r="G16" s="19"/>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A17" s="39"/>
+      <c r="B17" s="36"/>
+      <c r="C17" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="D17" s="15" t="s">
+        <v>58</v>
+      </c>
+      <c r="E17" s="23"/>
+      <c r="F17" s="16"/>
+      <c r="G17" s="19"/>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A18" s="39"/>
+      <c r="B18" s="36"/>
+      <c r="C18" s="35" t="s">
+        <v>14</v>
+      </c>
+      <c r="D18" s="15"/>
+      <c r="E18" s="15"/>
+      <c r="F18" s="15"/>
+      <c r="G18" s="19"/>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A19" s="39"/>
+      <c r="B19" s="36"/>
+      <c r="C19" s="36"/>
+      <c r="D19" s="15"/>
+      <c r="E19" s="15"/>
+      <c r="F19" s="15"/>
+      <c r="G19" s="19"/>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A20" s="39"/>
+      <c r="B20" s="36"/>
+      <c r="C20" s="36"/>
+      <c r="D20" s="15"/>
+      <c r="E20" s="15"/>
+      <c r="F20" s="15"/>
+      <c r="G20" s="19"/>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A21" s="39"/>
+      <c r="B21" s="36"/>
+      <c r="C21" s="37"/>
+      <c r="D21" s="19"/>
+      <c r="E21" s="19"/>
+      <c r="F21" s="19"/>
+      <c r="G21" s="19"/>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A22" s="39"/>
+      <c r="B22" s="36"/>
+      <c r="C22" s="35" t="s">
+        <v>15</v>
+      </c>
+      <c r="D22" s="19" t="s">
+        <v>91</v>
+      </c>
+      <c r="E22" s="16" t="s">
+        <v>133</v>
+      </c>
+      <c r="F22" s="16"/>
+      <c r="G22" s="19"/>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A23" s="39"/>
+      <c r="B23" s="36"/>
+      <c r="C23" s="36"/>
+      <c r="D23" s="20" t="s">
+        <v>98</v>
+      </c>
+      <c r="E23" s="14"/>
+      <c r="F23" s="14"/>
+      <c r="G23" s="19"/>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A24" s="39"/>
+      <c r="B24" s="36"/>
+      <c r="C24" s="36"/>
+      <c r="D24" s="21"/>
+      <c r="E24" s="21"/>
+      <c r="F24" s="21"/>
+      <c r="G24" s="19"/>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A25" s="39"/>
+      <c r="B25" s="37"/>
+      <c r="C25" s="37"/>
+      <c r="D25" s="21"/>
+      <c r="E25" s="21"/>
+      <c r="F25" s="21"/>
+      <c r="G25" s="19"/>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A26" s="39"/>
+      <c r="B26" s="35" t="s">
+        <v>16</v>
+      </c>
+      <c r="C26" s="35" t="s">
+        <v>24</v>
+      </c>
+      <c r="D26" s="21" t="s">
+        <v>110</v>
+      </c>
+      <c r="E26" s="26"/>
+      <c r="F26" s="26"/>
+      <c r="G26" s="19"/>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A27" s="39"/>
+      <c r="B27" s="36"/>
+      <c r="C27" s="36"/>
+      <c r="D27" s="21" t="s">
+        <v>111</v>
+      </c>
+      <c r="E27" s="26"/>
+      <c r="F27" s="26"/>
+      <c r="G27" s="19"/>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A28" s="39"/>
+      <c r="B28" s="36"/>
+      <c r="C28" s="36"/>
+      <c r="D28" s="21"/>
+      <c r="E28" s="21"/>
+      <c r="F28" s="21"/>
+      <c r="G28" s="19"/>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A29" s="39"/>
+      <c r="B29" s="36"/>
+      <c r="C29" s="35" t="s">
+        <v>25</v>
+      </c>
+      <c r="D29" s="21" t="s">
+        <v>79</v>
+      </c>
+      <c r="E29" s="26"/>
+      <c r="F29" s="26"/>
+      <c r="G29" s="19"/>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A30" s="39"/>
+      <c r="B30" s="36"/>
+      <c r="C30" s="36"/>
+      <c r="D30" s="21"/>
+      <c r="E30" s="21"/>
+      <c r="F30" s="21"/>
+      <c r="G30" s="19"/>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A31" s="39"/>
+      <c r="B31" s="36"/>
+      <c r="C31" s="37"/>
+      <c r="D31" s="21"/>
+      <c r="E31" s="21"/>
+      <c r="F31" s="21"/>
+      <c r="G31" s="19"/>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A32" s="39"/>
+      <c r="B32" s="36"/>
+      <c r="C32" s="35" t="s">
+        <v>26</v>
+      </c>
+      <c r="D32" s="21"/>
+      <c r="E32" s="21"/>
+      <c r="F32" s="21"/>
+      <c r="G32" s="19"/>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A33" s="39"/>
+      <c r="B33" s="36"/>
+      <c r="C33" s="36"/>
+      <c r="D33" s="21"/>
+      <c r="E33" s="21"/>
+      <c r="F33" s="21"/>
+      <c r="G33" s="19"/>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A34" s="39"/>
+      <c r="B34" s="36"/>
+      <c r="C34" s="36"/>
+      <c r="D34" s="21"/>
+      <c r="E34" s="21"/>
+      <c r="F34" s="21"/>
+      <c r="G34" s="19"/>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A35" s="39"/>
+      <c r="B35" s="36"/>
+      <c r="C35" s="37"/>
+      <c r="D35" s="21"/>
+      <c r="E35" s="21"/>
+      <c r="F35" s="21"/>
+      <c r="G35" s="19"/>
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A36" s="39"/>
+      <c r="B36" s="36"/>
+      <c r="C36" s="35" t="s">
+        <v>27</v>
+      </c>
+      <c r="D36" s="21" t="s">
+        <v>84</v>
+      </c>
+      <c r="E36" s="26"/>
+      <c r="F36" s="26"/>
+      <c r="G36" s="19"/>
+    </row>
+    <row r="37" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A37" s="39"/>
+      <c r="B37" s="36"/>
+      <c r="C37" s="37"/>
+      <c r="D37" s="21"/>
+      <c r="E37" s="21"/>
+      <c r="F37" s="21"/>
+      <c r="G37" s="19"/>
+    </row>
+    <row r="38" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A38" s="39"/>
+      <c r="B38" s="36"/>
+      <c r="C38" s="35" t="s">
+        <v>28</v>
+      </c>
+      <c r="D38" s="21" t="s">
+        <v>96</v>
+      </c>
+      <c r="E38" s="26"/>
+      <c r="F38" s="26"/>
+      <c r="G38" s="19"/>
+    </row>
+    <row r="39" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A39" s="39"/>
+      <c r="B39" s="36"/>
+      <c r="C39" s="36"/>
+      <c r="D39" s="21" t="s">
+        <v>97</v>
+      </c>
+      <c r="E39" s="26"/>
+      <c r="F39" s="26"/>
+      <c r="G39" s="19"/>
+    </row>
+    <row r="40" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A40" s="39"/>
+      <c r="B40" s="36"/>
+      <c r="C40" s="35" t="s">
+        <v>29</v>
+      </c>
+      <c r="D40" s="21" t="s">
+        <v>80</v>
+      </c>
+      <c r="E40" s="26"/>
+      <c r="F40" s="26"/>
+      <c r="G40" s="19"/>
+    </row>
+    <row r="41" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A41" s="39"/>
+      <c r="B41" s="36"/>
+      <c r="C41" s="36"/>
+      <c r="D41" s="21" t="s">
+        <v>81</v>
+      </c>
+      <c r="E41" s="26"/>
+      <c r="F41" s="26"/>
+      <c r="G41" s="19"/>
+    </row>
+    <row r="42" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A42" s="39"/>
+      <c r="B42" s="36"/>
+      <c r="C42" s="37"/>
+      <c r="D42" s="21" t="s">
+        <v>82</v>
+      </c>
+      <c r="E42" s="26"/>
+      <c r="F42" s="26"/>
+      <c r="G42" s="19"/>
+    </row>
+    <row r="43" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A43" s="39"/>
+      <c r="B43" s="36"/>
+      <c r="C43" s="35" t="s">
+        <v>30</v>
+      </c>
+      <c r="D43" s="21" t="s">
+        <v>61</v>
+      </c>
+      <c r="E43" s="26"/>
+      <c r="F43" s="26"/>
+      <c r="G43" s="19"/>
+    </row>
+    <row r="44" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A44" s="39"/>
+      <c r="B44" s="36"/>
+      <c r="C44" s="36"/>
+      <c r="D44" s="21" t="s">
+        <v>62</v>
+      </c>
+      <c r="E44" s="26"/>
+      <c r="F44" s="26"/>
+      <c r="G44" s="19"/>
+    </row>
+    <row r="45" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A45" s="39"/>
+      <c r="B45" s="36"/>
+      <c r="C45" s="37"/>
+      <c r="D45" s="21"/>
+      <c r="E45" s="21"/>
+      <c r="F45" s="21"/>
+      <c r="G45" s="19"/>
+    </row>
+    <row r="46" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A46" s="39"/>
+      <c r="B46" s="36"/>
+      <c r="C46" s="35" t="s">
+        <v>31</v>
+      </c>
+      <c r="D46" s="21"/>
+      <c r="E46" s="21"/>
+      <c r="F46" s="21"/>
+      <c r="G46" s="19"/>
+    </row>
+    <row r="47" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A47" s="39"/>
+      <c r="B47" s="36"/>
+      <c r="C47" s="36"/>
+      <c r="D47" s="21"/>
+      <c r="E47" s="21"/>
+      <c r="F47" s="21"/>
+      <c r="G47" s="19"/>
+    </row>
+    <row r="48" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A48" s="39"/>
+      <c r="B48" s="36"/>
+      <c r="C48" s="35" t="s">
+        <v>32</v>
+      </c>
+      <c r="D48" s="21" t="s">
+        <v>72</v>
+      </c>
+      <c r="E48" s="26"/>
+      <c r="F48" s="26"/>
+      <c r="G48" s="19"/>
+    </row>
+    <row r="49" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A49" s="39"/>
+      <c r="B49" s="36"/>
+      <c r="C49" s="36"/>
+      <c r="D49" s="21" t="s">
+        <v>73</v>
+      </c>
+      <c r="E49" s="26"/>
+      <c r="F49" s="26"/>
+      <c r="G49" s="19"/>
+    </row>
+    <row r="50" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A50" s="39"/>
+      <c r="B50" s="36"/>
+      <c r="C50" s="36"/>
+      <c r="D50" s="21"/>
+      <c r="E50" s="21"/>
+      <c r="F50" s="21"/>
+      <c r="G50" s="19"/>
+    </row>
+    <row r="51" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A51" s="39"/>
+      <c r="B51" s="36"/>
+      <c r="C51" s="35" t="s">
+        <v>33</v>
+      </c>
+      <c r="D51" s="21" t="s">
+        <v>112</v>
+      </c>
+      <c r="E51" s="26"/>
+      <c r="F51" s="26"/>
+      <c r="G51" s="19"/>
+    </row>
+    <row r="52" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A52" s="39"/>
+      <c r="B52" s="36"/>
+      <c r="C52" s="36"/>
+      <c r="D52" s="21"/>
+      <c r="E52" s="21"/>
+      <c r="F52" s="21"/>
+      <c r="G52" s="19"/>
+    </row>
+    <row r="53" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A53" s="39"/>
+      <c r="B53" s="36"/>
+      <c r="C53" s="36"/>
+      <c r="D53" s="21"/>
+      <c r="E53" s="21"/>
+      <c r="F53" s="21"/>
+      <c r="G53" s="19"/>
+    </row>
+    <row r="54" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A54" s="39"/>
+      <c r="B54" s="36"/>
+      <c r="C54" s="35" t="s">
+        <v>34</v>
+      </c>
+      <c r="D54" s="21" t="s">
+        <v>113</v>
+      </c>
+      <c r="E54" s="26"/>
+      <c r="F54" s="26"/>
+      <c r="G54" s="19"/>
+    </row>
+    <row r="55" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A55" s="39"/>
+      <c r="B55" s="36"/>
+      <c r="C55" s="37"/>
+      <c r="D55" s="21"/>
+      <c r="E55" s="21"/>
+      <c r="F55" s="21"/>
+      <c r="G55" s="19"/>
+    </row>
+    <row r="56" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A56" s="39"/>
+      <c r="B56" s="36"/>
+      <c r="C56" s="35" t="s">
+        <v>35</v>
+      </c>
+      <c r="D56" s="21" t="s">
+        <v>120</v>
+      </c>
+      <c r="E56" s="26"/>
+      <c r="F56" s="26"/>
+      <c r="G56" s="19"/>
+    </row>
+    <row r="57" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A57" s="39"/>
+      <c r="B57" s="37"/>
+      <c r="C57" s="36"/>
+      <c r="D57" s="21" t="s">
+        <v>121</v>
+      </c>
+      <c r="E57" s="26"/>
+      <c r="F57" s="26"/>
+      <c r="G57" s="19"/>
+    </row>
+    <row r="58" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A58" s="39"/>
+      <c r="B58" s="35" t="s">
+        <v>17</v>
+      </c>
+      <c r="C58" s="35" t="s">
+        <v>36</v>
+      </c>
+      <c r="D58" s="15" t="s">
+        <v>94</v>
+      </c>
+      <c r="E58" s="23"/>
+      <c r="F58" s="16"/>
+      <c r="G58" s="19"/>
+    </row>
+    <row r="59" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A59" s="39"/>
+      <c r="B59" s="36"/>
+      <c r="C59" s="36"/>
+      <c r="D59" s="15"/>
+      <c r="E59" s="15"/>
+      <c r="F59" s="16"/>
+      <c r="G59" s="19"/>
+    </row>
+    <row r="60" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A60" s="39"/>
+      <c r="B60" s="36"/>
+      <c r="C60" s="35" t="s">
+        <v>37</v>
+      </c>
+      <c r="D60" s="15" t="s">
+        <v>64</v>
+      </c>
+      <c r="E60" s="23"/>
+      <c r="F60" s="16"/>
+      <c r="G60" s="19"/>
+    </row>
+    <row r="61" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A61" s="39"/>
+      <c r="B61" s="36"/>
+      <c r="C61" s="36"/>
+      <c r="D61" s="15" t="s">
+        <v>65</v>
+      </c>
+      <c r="E61" s="23"/>
+      <c r="F61" s="16"/>
+      <c r="G61" s="19"/>
+    </row>
+    <row r="62" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A62" s="39"/>
+      <c r="B62" s="36"/>
+      <c r="C62" s="36"/>
+      <c r="D62" s="15" t="s">
+        <v>66</v>
+      </c>
+      <c r="E62" s="23"/>
+      <c r="F62" s="16"/>
+      <c r="G62" s="19"/>
+    </row>
+    <row r="63" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A63" s="39"/>
+      <c r="B63" s="36"/>
+      <c r="C63" s="36"/>
+      <c r="D63" s="15" t="s">
+        <v>67</v>
+      </c>
+      <c r="E63" s="23"/>
+      <c r="F63" s="16"/>
+      <c r="G63" s="19"/>
+    </row>
+    <row r="64" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A64" s="39"/>
+      <c r="B64" s="36"/>
+      <c r="C64" s="36"/>
+      <c r="D64" s="15" t="s">
+        <v>68</v>
+      </c>
+      <c r="E64" s="23"/>
+      <c r="F64" s="16"/>
+      <c r="G64" s="19"/>
+    </row>
+    <row r="65" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A65" s="39"/>
+      <c r="B65" s="36"/>
+      <c r="C65" s="36"/>
+      <c r="D65" s="15" t="s">
+        <v>69</v>
+      </c>
+      <c r="E65" s="23"/>
+      <c r="F65" s="16"/>
+      <c r="G65" s="19"/>
+    </row>
+    <row r="66" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A66" s="39"/>
+      <c r="B66" s="35" t="s">
+        <v>18</v>
+      </c>
+      <c r="C66" s="35" t="s">
+        <v>38</v>
+      </c>
+      <c r="D66" s="15" t="s">
+        <v>99</v>
+      </c>
+      <c r="E66" s="23"/>
+      <c r="F66" s="16"/>
+      <c r="G66" s="19"/>
+    </row>
+    <row r="67" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A67" s="39"/>
+      <c r="B67" s="36"/>
+      <c r="C67" s="36"/>
+      <c r="D67" s="15" t="s">
+        <v>100</v>
+      </c>
+      <c r="E67" s="23"/>
+      <c r="F67" s="16"/>
+      <c r="G67" s="19"/>
+    </row>
+    <row r="68" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A68" s="39"/>
+      <c r="B68" s="36"/>
+      <c r="C68" s="36"/>
+      <c r="D68" s="15" t="s">
+        <v>101</v>
+      </c>
+      <c r="E68" s="23"/>
+      <c r="F68" s="16"/>
+      <c r="G68" s="19"/>
+    </row>
+    <row r="69" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A69" s="39"/>
+      <c r="B69" s="36"/>
+      <c r="C69" s="35" t="s">
+        <v>39</v>
+      </c>
+      <c r="D69" s="15" t="s">
+        <v>74</v>
+      </c>
+      <c r="E69" s="23"/>
+      <c r="F69" s="16"/>
+      <c r="G69" s="19"/>
+    </row>
+    <row r="70" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A70" s="39"/>
+      <c r="B70" s="36"/>
+      <c r="C70" s="36"/>
+      <c r="D70" s="15" t="s">
+        <v>75</v>
+      </c>
+      <c r="E70" s="23"/>
+      <c r="F70" s="16"/>
+      <c r="G70" s="19"/>
+    </row>
+    <row r="71" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A71" s="39"/>
+      <c r="B71" s="36"/>
+      <c r="C71" s="36"/>
+      <c r="D71" s="15" t="s">
+        <v>76</v>
+      </c>
+      <c r="E71" s="23"/>
+      <c r="F71" s="16"/>
+      <c r="G71" s="19"/>
+    </row>
+    <row r="72" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A72" s="39"/>
+      <c r="B72" s="36"/>
+      <c r="C72" s="35" t="s">
+        <v>40</v>
+      </c>
+      <c r="D72" s="15" t="s">
+        <v>103</v>
+      </c>
+      <c r="E72" s="23"/>
+      <c r="F72" s="16"/>
+      <c r="G72" s="19"/>
+    </row>
+    <row r="73" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A73" s="39"/>
+      <c r="B73" s="36"/>
+      <c r="C73" s="36"/>
+      <c r="D73" s="15" t="s">
+        <v>104</v>
+      </c>
+      <c r="E73" s="23"/>
+      <c r="F73" s="16"/>
+      <c r="G73" s="19"/>
+    </row>
+    <row r="74" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A74" s="39"/>
+      <c r="B74" s="36"/>
+      <c r="C74" s="36"/>
+      <c r="D74" s="15" t="s">
+        <v>105</v>
+      </c>
+      <c r="E74" s="23"/>
+      <c r="F74" s="16"/>
+      <c r="G74" s="19"/>
+    </row>
+    <row r="75" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A75" s="39"/>
+      <c r="B75" s="36"/>
+      <c r="C75" s="36"/>
+      <c r="D75" s="15" t="s">
+        <v>106</v>
+      </c>
+      <c r="E75" s="23"/>
+      <c r="F75" s="16"/>
+      <c r="G75" s="19"/>
+    </row>
+    <row r="76" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A76" s="39"/>
+      <c r="B76" s="36"/>
+      <c r="C76" s="35" t="s">
+        <v>41</v>
+      </c>
+      <c r="D76" s="15" t="s">
+        <v>114</v>
+      </c>
+      <c r="E76" s="23"/>
+      <c r="F76" s="16"/>
+      <c r="G76" s="19"/>
+    </row>
+    <row r="77" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A77" s="39"/>
+      <c r="B77" s="36"/>
+      <c r="C77" s="36"/>
+      <c r="D77" s="15" t="s">
+        <v>115</v>
+      </c>
+      <c r="E77" s="23"/>
+      <c r="F77" s="16"/>
+      <c r="G77" s="19"/>
+    </row>
+    <row r="78" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A78" s="39"/>
+      <c r="B78" s="36"/>
+      <c r="C78" s="35" t="s">
+        <v>42</v>
+      </c>
+      <c r="D78" s="15" t="s">
+        <v>134</v>
+      </c>
+      <c r="E78" s="23"/>
+      <c r="F78" s="16"/>
+      <c r="G78" s="19"/>
+    </row>
+    <row r="79" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A79" s="39"/>
+      <c r="B79" s="36"/>
+      <c r="C79" s="36"/>
+      <c r="D79" s="15" t="s">
+        <v>124</v>
+      </c>
+      <c r="E79" s="23"/>
+      <c r="F79" s="16"/>
+      <c r="G79" s="19"/>
+    </row>
+    <row r="80" spans="1:7" ht="15.5" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A80" s="39"/>
+      <c r="B80" s="35" t="s">
+        <v>19</v>
+      </c>
+      <c r="C80" s="35" t="s">
+        <v>43</v>
+      </c>
+      <c r="D80" s="21" t="s">
+        <v>109</v>
+      </c>
+      <c r="E80" s="26"/>
+      <c r="F80" s="26"/>
+      <c r="G80" s="19"/>
+    </row>
+    <row r="81" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A81" s="39"/>
+      <c r="B81" s="36"/>
+      <c r="C81" s="37"/>
+      <c r="D81" s="15"/>
+      <c r="E81" s="15"/>
+      <c r="F81" s="15"/>
+      <c r="G81" s="19"/>
+    </row>
+    <row r="82" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A82" s="39"/>
+      <c r="B82" s="36"/>
+      <c r="C82" s="35" t="s">
+        <v>44</v>
+      </c>
+      <c r="D82" s="15" t="s">
+        <v>108</v>
+      </c>
+      <c r="E82" s="23"/>
+      <c r="F82" s="23"/>
+      <c r="G82" s="19"/>
+    </row>
+    <row r="83" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A83" s="39"/>
+      <c r="B83" s="37"/>
+      <c r="C83" s="37"/>
+      <c r="D83" s="15"/>
+      <c r="E83" s="15"/>
+      <c r="F83" s="15"/>
+      <c r="G83" s="19"/>
+    </row>
+    <row r="84" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A84" s="39"/>
+      <c r="B84" s="35" t="s">
+        <v>20</v>
+      </c>
+      <c r="C84" s="35" t="s">
+        <v>45</v>
+      </c>
+      <c r="D84" s="15" t="s">
+        <v>89</v>
+      </c>
+      <c r="E84" s="23"/>
+      <c r="F84" s="23"/>
+      <c r="G84" s="19"/>
+    </row>
+    <row r="85" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A85" s="39"/>
+      <c r="B85" s="36"/>
+      <c r="C85" s="36"/>
+      <c r="D85" s="15"/>
+      <c r="E85" s="15"/>
+      <c r="F85" s="15"/>
+      <c r="G85" s="19"/>
+    </row>
+    <row r="86" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A86" s="39"/>
+      <c r="B86" s="36"/>
+      <c r="C86" s="37"/>
+      <c r="D86" s="15"/>
+      <c r="E86" s="15"/>
+      <c r="F86" s="15"/>
+      <c r="G86" s="19"/>
+    </row>
+    <row r="87" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A87" s="39"/>
+      <c r="B87" s="36"/>
+      <c r="C87" s="35" t="s">
+        <v>46</v>
+      </c>
+      <c r="D87" s="15" t="s">
+        <v>128</v>
+      </c>
+      <c r="E87" s="23"/>
+      <c r="F87" s="23"/>
+      <c r="G87" s="19"/>
+    </row>
+    <row r="88" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A88" s="39"/>
+      <c r="B88" s="36"/>
+      <c r="C88" s="36"/>
+      <c r="D88" s="15"/>
+      <c r="E88" s="15"/>
+      <c r="F88" s="15"/>
+      <c r="G88" s="19"/>
+    </row>
+    <row r="89" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A89" s="39"/>
+      <c r="B89" s="36"/>
+      <c r="C89" s="35" t="s">
+        <v>47</v>
+      </c>
+      <c r="D89" s="15" t="s">
+        <v>78</v>
+      </c>
+      <c r="E89" s="23"/>
+      <c r="F89" s="23"/>
+      <c r="G89" s="19"/>
+    </row>
+    <row r="90" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A90" s="39"/>
+      <c r="B90" s="36"/>
+      <c r="C90" s="36"/>
+      <c r="D90" s="15"/>
+      <c r="E90" s="15"/>
+      <c r="F90" s="15"/>
+      <c r="G90" s="19"/>
+    </row>
+    <row r="91" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A91" s="39"/>
+      <c r="B91" s="36"/>
+      <c r="C91" s="35" t="s">
+        <v>48</v>
+      </c>
+      <c r="D91" s="15" t="s">
+        <v>77</v>
+      </c>
+      <c r="E91" s="23"/>
+      <c r="F91" s="23"/>
+      <c r="G91" s="19"/>
+    </row>
+    <row r="92" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A92" s="39"/>
+      <c r="B92" s="36"/>
+      <c r="C92" s="36"/>
+      <c r="D92" s="15"/>
+      <c r="E92" s="15"/>
+      <c r="F92" s="15"/>
+      <c r="G92" s="19"/>
+    </row>
+    <row r="93" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A93" s="39"/>
+      <c r="B93" s="36"/>
+      <c r="C93" s="35" t="s">
+        <v>49</v>
+      </c>
+      <c r="D93" s="15" t="s">
+        <v>125</v>
+      </c>
+      <c r="E93" s="23"/>
+      <c r="F93" s="23"/>
+      <c r="G93" s="19"/>
+    </row>
+    <row r="94" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A94" s="39"/>
+      <c r="B94" s="36"/>
+      <c r="C94" s="36"/>
+      <c r="D94" s="15" t="s">
+        <v>126</v>
+      </c>
+      <c r="E94" s="23"/>
+      <c r="F94" s="23"/>
+      <c r="G94" s="19"/>
+    </row>
+    <row r="95" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A95" s="39"/>
+      <c r="B95" s="36"/>
+      <c r="C95" s="36"/>
+      <c r="D95" s="15" t="s">
+        <v>127</v>
+      </c>
+      <c r="E95" s="23"/>
+      <c r="F95" s="23"/>
+      <c r="G95" s="19"/>
+    </row>
+    <row r="96" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A96" s="39"/>
+      <c r="B96" s="36"/>
+      <c r="C96" s="36"/>
+      <c r="D96" s="15"/>
+      <c r="E96" s="15"/>
+      <c r="F96" s="15"/>
+      <c r="G96" s="19"/>
+    </row>
+    <row r="97" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A97" s="39"/>
+      <c r="B97" s="36"/>
+      <c r="C97" s="36"/>
+      <c r="D97" s="15"/>
+      <c r="E97" s="15"/>
+      <c r="F97" s="15"/>
+      <c r="G97" s="19"/>
+    </row>
+    <row r="98" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A98" s="39"/>
+      <c r="B98" s="35" t="s">
+        <v>21</v>
+      </c>
+      <c r="C98" s="35" t="s">
+        <v>50</v>
+      </c>
+      <c r="D98" s="15" t="s">
+        <v>70</v>
+      </c>
+      <c r="E98" s="23"/>
+      <c r="F98" s="23"/>
+      <c r="G98" s="19"/>
+    </row>
+    <row r="99" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A99" s="39"/>
+      <c r="B99" s="36"/>
+      <c r="C99" s="36"/>
+      <c r="D99" s="15" t="s">
+        <v>71</v>
+      </c>
+      <c r="E99" s="23"/>
+      <c r="F99" s="23"/>
+      <c r="G99" s="19"/>
+    </row>
+    <row r="100" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A100" s="39"/>
+      <c r="B100" s="36"/>
+      <c r="C100" s="36"/>
+      <c r="D100" s="15" t="s">
+        <v>83</v>
+      </c>
+      <c r="E100" s="23"/>
+      <c r="F100" s="23"/>
+      <c r="G100" s="19"/>
+    </row>
+    <row r="101" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A101" s="39"/>
+      <c r="B101" s="36"/>
+      <c r="C101" s="35" t="s">
+        <v>51</v>
+      </c>
+      <c r="D101" s="15" t="s">
+        <v>116</v>
+      </c>
+      <c r="E101" s="23"/>
+      <c r="F101" s="23"/>
+      <c r="G101" s="19"/>
+    </row>
+    <row r="102" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A102" s="39"/>
+      <c r="B102" s="36"/>
+      <c r="C102" s="36"/>
+      <c r="D102" s="15" t="s">
+        <v>117</v>
+      </c>
+      <c r="E102" s="23"/>
+      <c r="F102" s="23"/>
+      <c r="G102" s="19"/>
+    </row>
+    <row r="103" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A103" s="39"/>
+      <c r="B103" s="36"/>
+      <c r="C103" s="36"/>
+      <c r="D103" s="15" t="s">
+        <v>118</v>
+      </c>
+      <c r="E103" s="23"/>
+      <c r="F103" s="23"/>
+      <c r="G103" s="19"/>
+    </row>
+    <row r="104" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A104" s="39"/>
+      <c r="B104" s="36"/>
+      <c r="C104" s="36"/>
+      <c r="D104" s="15" t="s">
+        <v>119</v>
+      </c>
+      <c r="E104" s="23"/>
+      <c r="F104" s="23"/>
+      <c r="G104" s="19"/>
+    </row>
+    <row r="105" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A105" s="39"/>
+      <c r="B105" s="36"/>
+      <c r="C105" s="35" t="s">
+        <v>52</v>
+      </c>
+      <c r="D105" s="15" t="s">
+        <v>122</v>
+      </c>
+      <c r="E105" s="23"/>
+      <c r="F105" s="23"/>
+      <c r="G105" s="19"/>
+    </row>
+    <row r="106" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A106" s="39"/>
+      <c r="B106" s="36"/>
+      <c r="C106" s="36"/>
+      <c r="D106" s="15"/>
+      <c r="E106" s="15"/>
+      <c r="F106" s="15"/>
+      <c r="G106" s="19"/>
+    </row>
+    <row r="107" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A107" s="39"/>
+      <c r="B107" s="36"/>
+      <c r="C107" s="13" t="s">
+        <v>53</v>
+      </c>
+      <c r="D107" s="15" t="s">
+        <v>86</v>
+      </c>
+      <c r="E107" s="23"/>
+      <c r="F107" s="23"/>
+      <c r="G107" s="19"/>
+    </row>
+    <row r="108" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A108" s="39"/>
+      <c r="B108" s="35" t="s">
+        <v>22</v>
+      </c>
+      <c r="C108" s="35" t="s">
+        <v>54</v>
+      </c>
+      <c r="D108" s="15" t="s">
+        <v>92</v>
+      </c>
+      <c r="E108" s="23"/>
+      <c r="F108" s="23"/>
+      <c r="G108" s="19"/>
+    </row>
+    <row r="109" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A109" s="39"/>
+      <c r="B109" s="36"/>
+      <c r="C109" s="37"/>
+      <c r="D109" s="15" t="s">
+        <v>93</v>
+      </c>
+      <c r="E109" s="23"/>
+      <c r="F109" s="23"/>
+      <c r="G109" s="19"/>
+    </row>
+    <row r="110" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A110" s="39"/>
+      <c r="B110" s="36"/>
+      <c r="C110" s="35" t="s">
+        <v>55</v>
+      </c>
+      <c r="D110" s="15" t="s">
+        <v>102</v>
+      </c>
+      <c r="E110" s="23"/>
+      <c r="F110" s="23"/>
+      <c r="G110" s="19"/>
+    </row>
+    <row r="111" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A111" s="39"/>
+      <c r="B111" s="37"/>
+      <c r="C111" s="37"/>
+      <c r="D111" s="15"/>
+      <c r="E111" s="15"/>
+      <c r="F111" s="15"/>
+      <c r="G111" s="19"/>
+    </row>
+    <row r="112" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A112" s="39"/>
+      <c r="B112" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="C112" s="11"/>
+      <c r="D112" s="15"/>
+      <c r="E112" s="15"/>
+      <c r="F112" s="15"/>
+      <c r="G112" s="19"/>
+    </row>
+    <row r="113" spans="1:8" x14ac:dyDescent="0.45">
+      <c r="A113" s="39"/>
+      <c r="B113" s="11"/>
+      <c r="C113" s="11"/>
+      <c r="D113" s="15"/>
+      <c r="E113" s="15"/>
+      <c r="F113" s="15"/>
+      <c r="G113" s="19"/>
+    </row>
+    <row r="114" spans="1:8" x14ac:dyDescent="0.45">
+      <c r="A114" s="39"/>
+      <c r="B114" s="11"/>
+      <c r="C114" s="11"/>
+      <c r="D114" s="15"/>
+      <c r="E114" s="15"/>
+      <c r="F114" s="15"/>
+      <c r="G114" s="19"/>
+    </row>
+    <row r="115" spans="1:8" x14ac:dyDescent="0.45">
+      <c r="A115" s="40"/>
+      <c r="B115" s="12"/>
+      <c r="C115" s="12"/>
+      <c r="D115" s="15"/>
+      <c r="E115" s="15"/>
+      <c r="F115" s="15"/>
+      <c r="G115" s="19"/>
+    </row>
+    <row r="116" spans="1:8" x14ac:dyDescent="0.45">
+      <c r="A116" s="39"/>
+      <c r="B116" s="41"/>
+      <c r="C116" s="28"/>
+      <c r="D116" s="19"/>
+      <c r="E116" s="19"/>
+      <c r="F116" s="19"/>
+      <c r="G116" s="19"/>
+    </row>
+    <row r="117" spans="1:8" x14ac:dyDescent="0.45">
+      <c r="A117" s="39"/>
+      <c r="B117" s="42"/>
+      <c r="C117" s="28"/>
+      <c r="D117" s="19"/>
+      <c r="E117" s="19"/>
+      <c r="F117" s="19"/>
+      <c r="G117" s="19"/>
+    </row>
+    <row r="118" spans="1:8" x14ac:dyDescent="0.45">
+      <c r="A118" s="39"/>
+      <c r="B118" s="43"/>
+      <c r="C118" s="28"/>
+      <c r="D118" s="19"/>
+      <c r="E118" s="19"/>
+      <c r="F118" s="19"/>
+      <c r="G118" s="19"/>
+      <c r="H118" s="9" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="119" spans="1:8" x14ac:dyDescent="0.45">
+      <c r="A119" s="39"/>
+      <c r="B119" s="41"/>
+      <c r="C119" s="28"/>
+      <c r="D119" s="19"/>
+      <c r="E119" s="19"/>
+      <c r="F119" s="16"/>
+      <c r="G119" s="19"/>
+    </row>
+    <row r="120" spans="1:8" x14ac:dyDescent="0.45">
+      <c r="A120" s="39"/>
+      <c r="B120" s="41"/>
+      <c r="C120" s="28"/>
+      <c r="D120" s="19"/>
+      <c r="E120" s="19"/>
+      <c r="F120" s="16"/>
+      <c r="G120" s="19"/>
+    </row>
+    <row r="121" spans="1:8" x14ac:dyDescent="0.45">
+      <c r="A121" s="39"/>
+      <c r="B121" s="41"/>
+      <c r="C121" s="28"/>
+      <c r="D121" s="19"/>
+      <c r="E121" s="19"/>
+      <c r="F121" s="16"/>
+      <c r="G121" s="19"/>
+    </row>
+    <row r="122" spans="1:8" x14ac:dyDescent="0.45">
+      <c r="A122" s="39"/>
+      <c r="B122" s="41"/>
+      <c r="C122" s="28"/>
+      <c r="D122" s="19"/>
+      <c r="E122" s="19"/>
+      <c r="F122" s="16"/>
+      <c r="G122" s="19"/>
+    </row>
+    <row r="123" spans="1:8" x14ac:dyDescent="0.45">
+      <c r="A123" s="39"/>
+      <c r="B123" s="41"/>
+      <c r="C123" s="28"/>
+      <c r="D123" s="19"/>
+      <c r="E123" s="19"/>
+      <c r="F123" s="19"/>
+      <c r="G123" s="19"/>
+    </row>
+    <row r="124" spans="1:8" x14ac:dyDescent="0.45">
+      <c r="A124" s="39"/>
+      <c r="B124" s="41"/>
+      <c r="C124" s="28"/>
+      <c r="D124" s="19"/>
+      <c r="E124" s="19"/>
+      <c r="F124" s="16"/>
+      <c r="G124" s="19"/>
+    </row>
+    <row r="125" spans="1:8" x14ac:dyDescent="0.45">
+      <c r="A125" s="39"/>
+      <c r="B125" s="41"/>
+      <c r="C125" s="28"/>
+      <c r="D125" s="19"/>
+      <c r="E125" s="19"/>
+      <c r="F125" s="19"/>
+      <c r="G125" s="19"/>
+    </row>
+    <row r="126" spans="1:8" x14ac:dyDescent="0.45">
+      <c r="A126" s="39"/>
+      <c r="B126" s="41"/>
+      <c r="C126" s="28"/>
+      <c r="D126" s="19"/>
+      <c r="E126" s="19"/>
+      <c r="F126" s="19"/>
+      <c r="G126" s="19"/>
+    </row>
+    <row r="127" spans="1:8" x14ac:dyDescent="0.45">
+      <c r="A127" s="39"/>
+      <c r="B127" s="41"/>
+      <c r="C127" s="28"/>
+      <c r="D127" s="19"/>
+      <c r="E127" s="19"/>
+      <c r="F127" s="19"/>
+      <c r="G127" s="19"/>
+    </row>
+    <row r="128" spans="1:8" x14ac:dyDescent="0.45">
+      <c r="A128" s="39"/>
+      <c r="B128" s="41"/>
+      <c r="C128" s="28"/>
+      <c r="D128" s="19"/>
+      <c r="E128" s="19"/>
+      <c r="F128" s="19"/>
+      <c r="G128" s="19"/>
+    </row>
+    <row r="129" spans="1:9" ht="17.5" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="A129" s="47"/>
+      <c r="B129" s="48"/>
+      <c r="C129" s="31"/>
+      <c r="D129" s="32"/>
+      <c r="E129" s="33"/>
+      <c r="F129" s="33"/>
+      <c r="G129" s="32"/>
+    </row>
+    <row r="131" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="I131" s="7"/>
+    </row>
+    <row r="132" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="I132" s="8"/>
+    </row>
+    <row r="133" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="I133" s="8"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="A4:G115" xr:uid="{34DC90E1-7112-4806-ADC5-98CA8498E977}"/>
+  <mergeCells count="49">
+    <mergeCell ref="A116:A129"/>
+    <mergeCell ref="B116:B117"/>
+    <mergeCell ref="B118:B129"/>
+    <mergeCell ref="B98:B107"/>
+    <mergeCell ref="C98:C100"/>
+    <mergeCell ref="C101:C104"/>
+    <mergeCell ref="C105:C106"/>
+    <mergeCell ref="B108:B111"/>
+    <mergeCell ref="C108:C109"/>
+    <mergeCell ref="C110:C111"/>
+    <mergeCell ref="B80:B83"/>
+    <mergeCell ref="C80:C81"/>
+    <mergeCell ref="C82:C83"/>
+    <mergeCell ref="B84:B97"/>
+    <mergeCell ref="C84:C86"/>
+    <mergeCell ref="C87:C88"/>
+    <mergeCell ref="C89:C90"/>
+    <mergeCell ref="C91:C92"/>
+    <mergeCell ref="C93:C97"/>
+    <mergeCell ref="B66:B79"/>
+    <mergeCell ref="C66:C68"/>
+    <mergeCell ref="C69:C71"/>
+    <mergeCell ref="C72:C75"/>
+    <mergeCell ref="C76:C77"/>
+    <mergeCell ref="C78:C79"/>
+    <mergeCell ref="C46:C47"/>
+    <mergeCell ref="C48:C50"/>
+    <mergeCell ref="C51:C53"/>
+    <mergeCell ref="C54:C55"/>
+    <mergeCell ref="C56:C57"/>
+    <mergeCell ref="B58:B65"/>
+    <mergeCell ref="C58:C59"/>
+    <mergeCell ref="C60:C65"/>
+    <mergeCell ref="C29:C31"/>
+    <mergeCell ref="C32:C35"/>
+    <mergeCell ref="C36:C37"/>
+    <mergeCell ref="C38:C39"/>
+    <mergeCell ref="C40:C42"/>
+    <mergeCell ref="C43:C45"/>
+    <mergeCell ref="A5:A115"/>
+    <mergeCell ref="B5:B11"/>
+    <mergeCell ref="C8:C9"/>
+    <mergeCell ref="C10:C11"/>
+    <mergeCell ref="B12:B25"/>
+    <mergeCell ref="C13:C15"/>
+    <mergeCell ref="C18:C21"/>
+    <mergeCell ref="C22:C25"/>
+    <mergeCell ref="B26:B57"/>
+    <mergeCell ref="C26:C28"/>
+  </mergeCells>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E2D875BA-B2A2-4199-A659-BF030CE3032F}">
+  <dimension ref="C2:H9"/>
+  <sheetFormatPr defaultRowHeight="17" x14ac:dyDescent="0.45"/>
+  <cols>
+    <col min="2" max="2" width="11.75" customWidth="1"/>
+    <col min="3" max="3" width="21.4140625" customWidth="1"/>
+    <col min="4" max="4" width="36.1640625" customWidth="1"/>
+    <col min="5" max="8" width="17.33203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="3:8" s="5" customFormat="1" x14ac:dyDescent="0.45">
+      <c r="E2" s="5" t="s">
+        <v>210</v>
+      </c>
+      <c r="F2" s="5" t="s">
+        <v>209</v>
+      </c>
+      <c r="G2" s="5" t="s">
+        <v>208</v>
+      </c>
+      <c r="H2" s="5" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="3" spans="3:8" s="5" customFormat="1" x14ac:dyDescent="0.45">
+      <c r="C3" s="5" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="4" spans="3:8" x14ac:dyDescent="0.45">
+      <c r="C4" t="s">
+        <v>212</v>
+      </c>
+      <c r="D4" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="5" spans="3:8" x14ac:dyDescent="0.45">
+      <c r="C5" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="9" spans="3:8" x14ac:dyDescent="0.45">
+      <c r="C9" s="5" t="s">
+        <v>64</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>